<commit_message>
Track iOS parity fixes and verification
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -449,10 +449,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr/>
-  <dimension ref="A1:S51"/>
-  <sheetViews/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:S57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1065,7 +1063,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>EntryCardDisplayMode.kt; EntryCard.kt; MainListViewModel.kt; ArchiveViewModel.kt</t>
+          <t>EntryCardDisplayMode.kt; EntryCard.kt; MainListViewModel.kt; ArchiveViewModel.kt; EntryCardDisplayModeStore.kt; RootView.swift; AppChrome.swift</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1075,7 +1073,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>表示モードが保存され、Main/Archiveで反映される。</t>
+          <t>表示モードが保存され、Main/Archive/Tag detailで反映される。AndroidはDataStore、iOSは@AppStorageで再起動後も保持する。</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1090,27 +1088,27 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests MainListViewModelTest.toggleEntryCardDisplayMode_updatesStore --tests ArchiveViewModelTest 成功。PASS: iOS generic simulator build成功。iOS RootView/AppChromeを@AppStorage保存へ修正。</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>物理Android/iPhoneでの表示モード切替と再起動後保持は未検証。以前のiOSは@Stateのみで再起動後保持しないギャップがあり、今回修正済み。</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>FIXED_LOCAL: iOS displayModeをEntryListDisplayMode.rawValue + @AppStorage("entryListDisplayMode")で永続化。</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>PASS local retest: Android targeted unit、iOS generic build成功。物理端末再起動保持は未実施。</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1125,12 +1123,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t/>
+          <t>iOS display mode persistence fixed 2026-06-29.</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 00:57:14 +0900</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1645,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>FetchMetadataWorker.kt; MetadataFetcher.kt; MetadataCoordinator.swift; MetadataStatusTextTests.swift; MetadataUiText.kt</t>
+          <t>FetchMetadataWorker.kt; MetadataFetcher.kt; MetadataCoordinator.swift; MetadataStatusTextTests.swift; MetadataUiText.kt; MetadataWorkScheduler.kt; ResolveWorker.kt; AppBackgroundScheduler.swift; BackgroundTaskRunner.swift</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1657,7 +1655,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>READY/PENDING/FAILED/UNAVAILABLEをUI文言へ分離し、部分成功をREADY扱いする。</t>
+          <t>READY/PENDING/FAILED/UNAVAILABLEをUI文言へ分離し、部分成功をREADY扱いする。 iOSはBGTaskSchedulerでbest-effortにmetadata backlogを再実行し、expiration時は一度だけ失敗完了する。</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1672,17 +1670,17 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: iOS MetadataStatusTextTests 5件成功し、BackgroundTaskRunnerの成功/失敗/expiration完了契約を確認。Android metadata系は既存unit/buildで通過済み。</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。 iOS実機BGTaskSchedulerの実スケジュール発火、Android WorkManager実機発火は未検証。</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1692,7 +1690,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>PASS local retest: iOS MetadataStatusTextTests成功。実機バックグラウンド発火は未実施。</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1707,12 +1705,12 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t/>
+          <t>iOS BGTaskScheduler/BackgroundTaskRunner coverage added 2026-06-29.</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 00:57:14 +0900</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2227,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>SharedTagSyncWorker.kt; SharedTagSyncCoordinator.kt; SharedTagSyncExecutor.swift; SharedTagCloud.swift</t>
+          <t>SharedTagSyncWorker.kt; SharedTagSyncCoordinator.kt; SharedTagSyncExecutor.swift; SharedTagCloud.swift; SQLiteDatabase.swift</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2254,27 +2252,27 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: iOS MetadataStatusTextTests 5件成功。SharedTagCloud migrationのdisplay_name追加をaddColumnIfMissingへ変更し、重複カラムログが消えたことを/tmp/rinbam-metadata-test.logで確認。</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>物理端末での共有タグ同期/グループ同期、Supabase live syncは未検証。iOS simulatorではApp Group entitlement警告とCoreSimulator WebCore/WebKit重複クラス警告が残るが、display_name重複カラムログは解消。</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>FIXED_LOCAL: SharedTagCloud migrationのtry? ALTER TABLEをSQLiteDatabase.addColumnIfMissingへ置換し、既存DBでの冪等性を改善。</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>PASS local retest: xcodebuild test -only-testing:URLSaveriOSTests/MetadataStatusTextTests 成功、重複display_name migrationログなし。</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2284,17 +2282,17 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>NOT VERIFIED on physical iPhone: 共有タグ/グループ同期は未検証。</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t/>
+          <t>iOS shared tag display_name migration idempotency fixed 2026-06-29.</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 01:02:48 +0900</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2324,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>DefaultTagRepository.kt; SharedTagCloudScreens.kt; SharedTagManagementSheets.swift; SharedTagCloud.swift</t>
+          <t>DefaultTagRepository.kt; SharedTagCloudScreens.kt; SharedTagManagementSheets.swift; SharedTagCloud.swift; SQLiteDatabase.swift</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2351,27 +2349,27 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: iOS MetadataStatusTextTests 5件成功。SharedTagCloud migrationのdisplay_name追加をaddColumnIfMissingへ変更し、重複カラムログが消えたことを/tmp/rinbam-metadata-test.logで確認。</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>物理端末での共有タグ同期/グループ同期、Supabase live syncは未検証。iOS simulatorではApp Group entitlement警告とCoreSimulator WebCore/WebKit重複クラス警告が残るが、display_name重複カラムログは解消。</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>FIXED_LOCAL: SharedTagCloud migrationのtry? ALTER TABLEをSQLiteDatabase.addColumnIfMissingへ置換し、既存DBでの冪等性を改善。</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>PASS local retest: xcodebuild test -only-testing:URLSaveriOSTests/MetadataStatusTextTests 成功、重複display_name migrationログなし。</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2381,17 +2379,17 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>NOT VERIFIED on physical iPhone: 共有タグ/グループ同期は未検証。</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t/>
+          <t>iOS shared tag display_name migration idempotency fixed 2026-06-29.</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 01:02:48 +0900</t>
         </is>
       </c>
     </row>
@@ -2714,7 +2712,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>EntitlementGrantRepository.kt; SharedTagCloudScreens.kt; URLSaverAppModel.swift; SharedTagCloud.swift</t>
+          <t>EntitlementGrantRepository.kt; SharedTagCloudScreens.kt; URLSaverAppModel.swift; SharedTagCloud.swift; EntitlementGrantStore.kt; EntitlementGrantRemoteDataSource.kt; UsageSummaryDataSource.kt</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2739,27 +2737,27 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests EntitlementResolverTest 成功。PASS: iOS URLRulesTests LimitChecker対象2件成功。SharedTagAuthViewModelTestは直近実行済み。</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>本番Supabase RPC/get_my_entitlement_grants/redeem_promo_code live実行、実メール/リンクからの優待適用、物理端末操作は未検証。</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>修正なし: ローカルテスト上のエラー未検出。Entitlement cache/remote/usage summaryのcode_basisを補強。</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>PASS local retest: Android entitlement targeted test、iOS limit checker targeted tests成功。</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2774,12 +2772,12 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t/>
+          <t>entitlement cache/remote coverage refreshed 2026-06-29.</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 01:00:20 +0900</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2809,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>PlanModels.kt; Models.swift; EntitlementResolver.kt</t>
+          <t>PlanModels.kt; Models.swift; EntitlementResolver.kt; UsageSummaryDataSource.kt; EntitlementResolverTest.kt; URLRulesTests.swift</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2836,27 +2834,27 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests EntitlementResolverTest 成功。PASS: iOS URLRulesTests LimitChecker対象2件成功。</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>物理端末で実使用量が上限に達した時のUI文言/ブロック、Supabase live grant反映は未検証。</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>修正なし: ローカル制限判定テスト上のエラー未検出。</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>PASS local retest: Android/iOS limit checker targeted tests成功。</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -2871,12 +2869,12 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t/>
+          <t>usage/limit checker coverage refreshed 2026-06-29.</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 01:00:20 +0900</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2906,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>ExportRepository.kt; ExportScreen.kt; ExportArchiveBuilder.swift; ExportSheet.swift</t>
+          <t>ExportRepository.kt; ExportScreen.kt; ExportArchiveBuilder.swift; ExportSheet.swift; ExportViewModel.kt; ActivityShareSheet.swift; URLSaverAppModel.swift</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2918,7 +2916,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>manifest、entries.jsonl、entries/*.md またはJSONを生成し、範囲/タグ/状態/サービス/メモ/日付フィルタ対応。</t>
+          <t>manifest、entries.jsonl、entries/*.md またはJSONを生成し、範囲/タグ/状態/サービス/メモ/日付フィルタ対応。Androidは共有シート/ファイル保存、iOSはUIActivityViewController/fileExporterで出力できる。</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2933,47 +2931,47 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests ExportRepositoryTest --tests ExportScreenTest 成功。PASS: iOS ExportArchiveBuilderTests/ServiceFilterTests 対象実行19件中Export関連17件成功。</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>物理Android/iPhoneでの共有シート、ファイル保存、ファイル受け渡し先アプリでの実確認は未検証。iOS simulator test中にApp Group entitlement警告と重複display_name migrationログあり、テスト失敗はなし。</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>修正なし: ローカルテスト上のエラー未検出。台帳code_basisに共有シート/保存先実装を補強。</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>PASS local retest: Android export targeted tests、iOS export/filter targeted tests成功。物理共有先は未実施。</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>未実機操作: export共有シート/ファイル保存は未検証。</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>NOT VERIFIED on physical iPhone: export共有シート/fileExporterは未検証。</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t/>
+          <t>export share/file destination coverage refreshed 2026-06-29.</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 01:00:20 +0900</t>
         </is>
       </c>
     </row>
@@ -4132,12 +4130,12 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>US-034/US-035/US-036/AS-008/ES-006を追加。</t>
+          <t>US-034/US-035/US-036/AS-008/ES-006を追加。 US-037/US-038/US-039/US-040/TS-001を追加。 AS-009を追加し、US-039に公開reset-passwordページを追記。 US-006のiOS表示モード永続化ギャップを修正し、US-012にiOS BGTaskScheduler証跡を追記。 US-025/US-023/US-024のexport/entitlement近接テスト結果を更新。US-040にiOS PrivacyInfo証跡を補強。 iOS SharedTagCloud display_name migrationの冪等性を修正し、US-018/US-019/ES-003へ反映。</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>2026-06-29 00:43:50 +0900</t>
+          <t>2026-06-29 01:02:48 +0900</t>
         </is>
       </c>
     </row>
@@ -4291,27 +4289,27 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS_WITH_LIVE_SUPABASE_ENV_GAP</t>
+          <t>PARTIAL_PASS_WITH_CORE_SIMULATOR_WARNING</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>PASS: 2026-06-29 iOS generic Simulator build成功、URLRepositoryTests単独成功、PendingInviteStoreTests単独成功。PARTIAL: 全体XCTestはSharedTagCloudLiveSyncTests 3件がInvalid API keyで失敗。</t>
+          <t>PASS: iOS MetadataStatusTextTests 5件成功。display_name duplicate column migrationログとApp Group container_create_or_lookup警告は修正後に消失。</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>iOS全体XCTest: live Supabase shared-tag tests が Invalid API key で失敗。ローカル対象テストは成功。物理iPhone UI操作は未検証。</t>
+          <t>iOS simulator testでCoreSimulator WebCore/WebKit重複クラス警告は残存。物理iPhone UI操作は未検証。</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>PARTIAL_FIXED_LOCAL: SharedTagCloud migrationの重複カラムログとSharedContainerのXCTest時App Group lookup警告を修正。残る警告はCoreSimulator runtime由来として継続記録。</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>PASS local targeted retest。live Supabaseキー/環境が整ったら全体再実行。</t>
+          <t>PASS local retest: MetadataStatusTextTests成功、duplicate display_nameログなし、container_create_or_lookupログなし。</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -4326,12 +4324,12 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t/>
+          <t>App Group XCTest warning fixed 2026-06-29; CoreSimulator UIAccessibilityLoaderWebShared warning remains.</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>2026-06-29 00:36:46 +0900</t>
+          <t>2026-06-29 01:07:00 +0900</t>
         </is>
       </c>
     </row>
@@ -5399,6 +5397,588 @@
       <c r="S51" t="inlineStr">
         <is>
           <t>2026-06-29 00:43:50 +0900</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>US-037</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>ユーザー</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Android/iOS</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>一覧</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>保存リンク検索</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>UrlSaverRoot.kt; RootView.swift; MainListViewModel.kt; URLSaverAppModel.swift</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>ユーザーとして、保存済みリンクをタイトル、URL、ホスト、コレクション、タグ名で検索し、目的のリンクだけを一覧に絞り込める。</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>検索アイコンで検索欄を表示し、入力中はActive一覧が絞り込まれる。クリアまたは戻る操作で検索状態を解除し、使い方画面表示中の検索操作はホーム検索へ戻る。</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Android/iOS source inspection; future UI test: search input, clear, no-result, guide-to-search transition. Android existing local build/test/lint; iOS generic build.</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>正準Android/iOSアプリで実データを消さずに検索欄表示、入力、クリア、戻るが動くこと。</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>SOURCE_CONFIRMED_WITH_UI_TEST_GAP</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>PASS(source): Android filterEntriesBySearch and searchBarVisible, iOS isShowingSearchBar/searchQuery UIを確認。近接build/testは既存実行で成功済み。</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>専用unit/UIテストと物理端末検索操作は未実施。Androidの検索はprivate UI関数中心で現在はソース確認寄り。</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>修正なし: 台帳未記載の既存機能として追加。</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>未実施: 専用UI確認が必要。</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>未実機操作: 検索欄表示/入力/クリアは未検証。</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>NOT VERIFIED on physical iPhone: 検索欄表示/入力/クリアは未検証。</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>AS-005の管理者検索とは別のユーザー向けホーム検索。</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>2026-06-29 00:49:24 +0900</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>US-038</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>ユーザー</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Android/iOS</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>一覧</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>複数選択で一括アーカイブ/削除</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>UrlSaverRoot.kt; MainActivityViewModel.kt; RootView.swift; URLSaverAppModel.swift</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>ユーザーとして、複数の保存リンクを選択してまとめてアーカイブまたは削除し、Undoで戻せる。</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>選択モード、個別選択、すべて選択、キャンセル、一括アーカイブ、一括pending delete、Undo通知が動く。選択中は通常ボトムバーを隠す。</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Android/iOS source inspection; Android targeted unit for MainActivityViewModel batch archive/delete; iOS source inspection for archive(entryIDs)/markPendingDelete(entryIDs). Future physical UI selection.</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>実データ保護のため物理端末ではテスト用データで選択/Undoまで確認すること。</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>SOURCE_CONFIRMED_WITH_DEVICE_GAP</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>PASS(source): Android selectedEntryIds/EntrySelectionBar/archiveEntries/markPendingDeleteEntries確認。iOS EntrySelectionBar/archive(entryIDs)/markPendingDelete(entryIDs)確認。</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>物理端末UI操作と専用UIテスト未実施。</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>修正なし: 台帳未記載の既存機能として追加。</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>未実施: UI実操作確認が必要。</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>未実機操作: 一括選択/Undoは未検証。</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>NOT VERIFIED on physical iPhone: 一括選択/Undoは未検証。</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>US-007/US-008の単体操作とは別の一括操作。</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>2026-06-29 00:49:24 +0900</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>US-039</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ユーザー</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Android/iOS/Supabase</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>プロフィール</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>確認メール再送/パスワード再設定</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>SharedTagCloudScreens.kt; SharedTagAuthViewModel.kt; DefaultTagRepository.kt; SharedTagAuthRemoteDataSource.kt; SharedTagCloudSheet.swift; URLSaverAppModel.swift; SharedTagCloud.swift; web/invite-link/auth/reset-password/index.html; web/invite-link/index.html; web/invite-link/vercel.json</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>ユーザーとして、共有タグクラウドのサインイン/招待参加で確認メールを再送したり、パスワード再設定メールを送信できる。</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>メール入力後、確認メール再送とパスワード再設定ボタンがSupabase auth endpointを呼び、成功/失敗メッセージを表示する。招待参加画面でも同じ補助導線を使える。 公開reset-passwordページはSupabase recovery code/sessionを受け取り、8文字以上かつ確認一致後にupdateUserで新パスワードを設定する。</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Android SharedTagAuthViewModelTest/TagRepositoryTest source; iOS source inspection/generic build; future Supabase auth live mail delivery verification.</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>本番Supabase auth SMTP/redirect URL設定で実メールが届き、アプリの文言が成功扱いだけで誤解を生まないこと。</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_MAIL_GAP</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>PASS: ./gradlew testDebugUnitTest --tests SharedTagAuthViewModelTest 成功。Source inspectionでAndroid/iOS resendEmailConfirmation/sendPasswordRecovery経路確認。 PASS(source): reset-password static pageのexchangeCodeForSession/updateUser/signOut経路を確認。</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Supabase本番メール送信/到達、redirect挙動、物理端末操作は未検証。 公開reset-passwordページのlive到達と実メールリンクからの更新は未検証。</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>修正なし: US-020から独立した補助機能として台帳追加。</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>未実施: live auth mailが必要。</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>未実機操作: 確認メール再送/パスワード再設定は未検証。</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>NOT VERIFIED on physical iPhone: 確認メール再送/パスワード再設定は未検証。</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>US-020は基本サインイン系。メール補助は外部メール到達が別ゲート。 targeted unit pass 2026-06-29. reset-password public page source-confirmed 2026-06-29.</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>2026-06-29 00:52:34 +0900</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>US-040</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ユーザー</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Android/Store</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>プライバシー/広告</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>データ取り扱い表示と広告無効化ガード</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>UrlSaverRoot.kt; strings.xml; AdsConfig.kt; AdsManager.kt; BannerAdSlot.kt; AdsConfigTest.kt; docs/release/final-submission-checklist.md; ios/URLSaveriOS/PrivacyInfo.xcprivacy; ios/URLSaverShareExtension/PrivacyInfo.xcprivacy</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>ユーザーとして、保存データの扱いをアプリ内で確認でき、リリース設定では広告SDKが初期化/表示されない状態で使える。</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>プライバシーダイアログ文言が表示可能で、ADS_ENABLED/ADS_TRIAL_LAUNCH_ADS_ENABLEDが無効ならSDK初期化、バナー、インタースティシャルが走らない。</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Android AdsConfigTest; source inspection for privacy dialog; release checklist review; future physical UI privacy dialog確認。</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Google Playのデータセーフティ/広告申告、リリースmanifest、アプリ内説明が最終build設定と一致すること。</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>LOCAL_PASS_WITH_STORE_DECLARATION_GAP</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>PASS: ./gradlew testDebugUnitTest --tests AdsConfigTest 成功。Source inspectionでprivacy_dialog stringsとUrlSaverRoot AlertDialogを確認。</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>物理端末でのプライバシーダイアログ表示とPlay Console最終申告一致は未検証。</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>修正なし: 台帳未記載の既存ユーザー/ストア影響機能として追加。</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>未実施: store申告最終確認が必要。</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>未実機操作: プライバシーダイアログ表示は未検証。</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>ES-006は公開Web/リンク。これはAndroidアプリ内表示と広告ガード。 targeted unit pass 2026-06-29. iOS privacy manifests included in release source review.</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>2026-06-29 01:00:20 +0900</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>TS-001</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>開発/従業員</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Android</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>未実装基盤</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>UserLabel DB/Repository基盤のみでUI未接続</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>UserLabelDao.kt; RoomModels.kt; AppDatabase.kt; DefaultUrlRepositoryCollectionsSupport.kt; UrlRepository.kt; MigrationDedupTest.kt</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>開発者として、将来のユーザーラベル機能のDB/Repository基盤がある一方、現行アップロード対象アプリではユーザーがラベルを作成/割当/削除するUIが未提供であることを追跡できる。</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>user_labels table、url_entries.userLabelId、create/delete/assign API、migration testが存在する。Compose/SwiftUIのユーザー操作面には同等ラベルUIがないことを明示する。</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Android source inspection; MigrationDedupTest migration_8_9_preservesExistingData_andCreatesUserLabels; rgでUI参照確認。</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>リリース判断時に「基礎はあるがユーザー機能ではない」と扱い、ストア説明やUI期待に載せないこと。</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>FOUNDATION_ONLY_NOT_USER_FACING</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>PASS: ./gradlew testDebugUnitTest --tests MigrationDedupTest.migration_8_9_preservesExistingData_andCreatesUserLabels 成功。DAO/Entity/Repository/APIはsource確認、UI入口は未確認。</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>機能基礎はあるが現行ユーザーUI未実装。iOS側に同等UserLabelモデルは未確認。</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>未修正: 仕様化するならAndroid UI追加とiOS parity設計が必要。現状は未実装基盤として記録。</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>未実施: UI実装後に再テスト。</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>該当UIなし。</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>該当UIなし。</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>ユーザー依頼の「基礎は作ったが実装していないもの」候補として追跡。 targeted unit pass 2026-06-29.</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>2026-06-29 00:50:01 +0900</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>AS-009</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>管理者</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Web/Admin/Resend</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>配信監査</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Resend message id手動配送照会</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>web/admin/app/api/admin/promo-codes/[id]/delivery/route.ts; web/admin/app/page.tsx; web/admin/lib/auth.ts; web/admin/lib/env.ts</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>管理者として、優待コードに保存されたResend message idからResend APIを照会し、最後の配送イベントや宛先情報を確認できる。</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>管理者認証が必要。delivery_message_idがない場合は404を返し、Resend API応答からid/message_id/from/to/subject/created_at/last_eventを返す。RESEND_API_KEY未設定やResendエラーは明示する。</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Web admin npm typecheck/build; source inspection; future live Resend API call with real delivery_message_id.</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>本番管理者トークン、service role、RESEND_API_KEY、実delivery_message_idでResendのtruthとDB状態が一致すること。</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>LOCAL_PASS_WITH_RESEND_LIVE_GAP</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>PASS: npm run typecheck &amp;&amp; npm run build 成功。Next build route一覧に /api/admin/promo-codes/[id]/delivery が含まれることを確認。Source inspectionでResend API照会経路確認。</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Resend live API照会、実message id、管理画面ボタン/表示の操作は未検証。</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>修正なし: AS-006 webhook追跡とは別の手動配送照会機能として台帳追加。</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>未実施: live Resend APIと管理者セッションが必要。</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>AS-006はwebhook反映、AS-009はResend APIへの手動照会。</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>2026-06-29 00:53:06 +0900</t>
         </is>
       </c>
     </row>
@@ -5408,105 +5988,271 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr/>
-  <dimension ref="A1:B8"/>
-  <sheetViews/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>項目</t>
+          <t>status</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>値</t>
+          <t>count</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>更新日時</t>
+          <t>ANDROID_LOCAL_PASS_WITH_IOS_MODEL_DIFFERENCE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-29 00:43:50 +0900</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>総ストーリー数</t>
+          <t>DOCUMENTED_PASS_WITH_FINAL_SHA_GAP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>今回追加</t>
+          <t>FOUNDATION_ONLY_NOT_USER_FACING</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>US-034 共有保存時タグ選択/作成, US-035 コレクション, US-036 ChatGPT sync, AS-008 問い合わせ監査, ES-006 公開Web/リンク</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Android targeted</t>
+          <t>LOCAL_PASS: Web build/typecheck成功。本番DB/API実動作は未検証</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PASS: ShareReceiverActivityEntrypointTest/RepositoryBehaviorTest/MainListViewModelTest/ListFilterStateTest/TopFilterOrderResolutionTest; ContactSupportClientTest</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Supabase functions</t>
+          <t>LOCAL_PASS_WITH_DEPLOY_GAP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PASS: deno check verify-store-purchase/contact-support/contact-support-resend-webhook</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Known gaps</t>
+          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Physical share/invite/purchase operations, Supabase DB live/RLS, store sandbox purchases, final Play SHA remain unverified</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>未コミット注意</t>
+          <t>LOCAL_PASS_WITH_EXTERNAL_STORE_GAP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>build.gradle.kts remains uncommitted unrelated AGP version change</t>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LOCAL_PASS_WITH_RESEND_LIVE_GAP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LOCAL_PASS_WITH_STORE_DECLARATION_GAP</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_LIVE_GAP</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_MAIL_GAP</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PARTIAL_PASS: Android実機PASS、iPhone UI操作は未検証</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PARTIAL_PASS: Android実機PASS、iPhone launchのみPASS</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PARTIAL_PASS_WITH_LOCAL_DB_GAP</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PARTIAL_PASS_WITH_SIMULATOR_WARNINGS</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PASS: Androidローカル検証成功、release buildも成功、実機共有系は未検証</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PASS: Web管理画面 typecheck/build 成功</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PASS: 正準スプレッドシート/CSV更新済み</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SOURCE_CONFIRMED_WITH_DEVICE_GAP</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SOURCE_CONFIRMED_WITH_UI_TEST_GAP</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore tag and collection parity flows
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -5025,7 +5025,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Android</t>
+          <t>Android/iOS</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5040,7 +5040,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>CollectionDao.kt; CollectionModels.kt; DefaultUrlRepositoryCollectionsSupport.kt; CollectionFilterRow.kt; MainListViewModel.kt; RepositoryBehaviorTest.kt; TopFilterOrderResolutionTest.kt</t>
+          <t>CollectionDao.kt; CollectionModels.kt; DefaultUrlRepositoryCollectionsSupport.kt; CollectionFilterRow.kt; MainListViewModel.kt; URLRepository.swift; Models.swift; URLRepositoryTests.swift</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>RepositoryBehaviorTest; MainListViewModelTest; ListFilterStateTest; TopFilterOrderResolutionTest; assembleDebug/testDebugUnitTest/lintDebug</t>
+          <t>Android: RepositoryBehaviorTest/MainListViewModelTest/ListFilterStateTest/TopFilterOrderResolutionTest. iOS: URLRepositoryTests collection lifecycle. Future iOS collection UI tests.</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5065,27 +5065,27 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>ANDROID_LOCAL_PASS_WITH_IOS_MODEL_DIFFERENCE</t>
+          <t>LOCAL_PASS_WITH_IOS_UI_GAP</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>PASS: RepositoryBehaviorTest/MainListViewModelTest/ListFilterStateTest/TopFilterOrderResolutionTest対象実行成功。Android全体build/test/lint成功。</t>
+          <t>PASS: Android RepositoryBehaviorTest/MainListViewModelTest/ListFilterStateTest/TopFilterOrderResolutionTest対象実行成功。PASS: iOS URLRepositoryTests 12件成功、受信箱/作成/重複/移動/並び替え/削除時受信箱戻しを確認。</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>iOSは同名のcollectionモデルではなくlocal tag中心の整理UI。Android固有機能として記録。物理Androidで並び替え/削除は未検証。</t>
+          <t>iOSはcollectionsテーブル/API/URLRecord.collectionIDの土台を追加済み。自作コレクションの作成、移動、並び替え、フィルタUIは未実装。物理Androidで並び替え/削除は未検証。</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>修正なし: ローカルテスト上のエラー未検出。</t>
+          <t>PARTIAL_FIXED_LOCAL: iOS collectionsテーブル、CollectionSummary、create/assign/reorder/delete/load API、collection_id DEFAULT 1を追加。US-035完全復元にはiOS UI接続が必要。</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>PASS local retest。実機UI操作は未実施。</t>
+          <t>PASS local retest: iOS URLRepositoryTests 12件成功。Android既存ローカルテストは前回成功済み。iOS UI実装/実機操作は未実施。</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5095,17 +5095,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t/>
+          <t>NOT VERIFIED on physical iPhone: コレクション作成/移動/並び替え/フィルタUIは未実装・未検証。</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>iOS parityはlocal tag管理で別途US-014/US-031/US-034に追跡。</t>
+          <t>iOS collection repository/API foundation added 2026-06-29; full UI parity still required.</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>2026-06-29 00:43:50 +0900</t>
+          <t>2026-06-29 01:24:00 +0900</t>
         </is>
       </c>
     </row>
@@ -5428,7 +5428,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>UrlSaverRoot.kt; RootView.swift; MainListViewModel.kt; URLSaverAppModel.swift</t>
+          <t>UrlSaverRoot.kt; MainListViewModel.kt; TagDao.kt; RootView.swift; ServiceFilterTests.swift; MainListViewModelTest.kt</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -5438,12 +5438,12 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>検索アイコンで検索欄を表示し、入力中はActive一覧が絞り込まれる。クリアまたは戻る操作で検索状態を解除し、使い方画面表示中の検索操作はホーム検索へ戻る。</t>
+          <t>検索アイコンで検索欄を表示し、入力中はActive一覧が絞り込まれる。Androidはタイトル/URL/ホスト/コレクション名/割当ローカルタグ名、iOSはタイトル/URL/ホスト/割当ローカルタグ名を検索対象にする。未割当タグ名ではヒットしない。</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Android/iOS source inspection; future UI test: search input, clear, no-result, guide-to-search transition. Android existing local build/test/lint; iOS generic build.</t>
+          <t>Android: MainListViewModelTest search tests. iOS: ServiceFilterTests search tests. Future UI test: search input, clear, no-result, guide-to-search transition.</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -5453,27 +5453,27 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>SOURCE_CONFIRMED_WITH_UI_TEST_GAP</t>
+          <t>LOCAL_PASS_WITH_UI_DEVICE_GAP</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>PASS(source): Android filterEntriesBySearch and searchBarVisible, iOS isShowingSearchBar/searchQuery UIを確認。近接build/testは既存実行で成功済み。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.MainListViewModelTest 成功。PASS: xcodebuild test -only-testing:URLSaveriOSTests/ServiceFilterTests 成功、15 tests。</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>専用unit/UIテストと物理端末検索操作は未実施。Androidの検索はprivate UI関数中心で現在はソース確認寄り。</t>
+          <t>物理Android/iPhoneでの検索欄表示、入力、クリア、戻る操作は未検証。iOSはcollections Repository/APIの土台は追加済みだが、RootView検索へのコレクション名連携はまだ未接続。</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>修正なし: 台帳未記載の既存機能として追加。</t>
+          <t>FIXED_LOCAL: Androidのタグ名検索が任意タグ名一致で全件ヒットし得る誤爆を修正。Android/iOSとも割当ローカルタグ名だけを検索対象にするテストを追加。</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>未実施: 専用UI確認が必要。</t>
+          <t>PASS local retest: Android MainListViewModelTest、iOS ServiceFilterTests 成功。UI実操作は未実施。</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -5488,12 +5488,12 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>AS-005の管理者検索とは別のユーザー向けホーム検索。</t>
+          <t>User search local-tag false-positive fixed 2026-06-29. iOS collection repository/API foundation exists; collection-name search still needs RootView/UI wiring.</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>2026-06-29 00:49:24 +0900</t>
+          <t>2026-06-29 01:24:30 +0900</t>
         </is>
       </c>
     </row>
@@ -5525,7 +5525,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>UrlSaverRoot.kt; MainActivityViewModel.kt; RootView.swift; URLSaverAppModel.swift</t>
+          <t>UrlSaverRoot.kt; MainListViewModel.kt; RootView.swift; URLSaverAppModel.swift; URLRepository.swift; MainListViewModelTest.kt; URLRepositoryTests.swift</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -5540,7 +5540,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Android/iOS source inspection; Android targeted unit for MainActivityViewModel batch archive/delete; iOS source inspection for archive(entryIDs)/markPendingDelete(entryIDs). Future physical UI selection.</t>
+          <t>Android: MainListViewModelTest batch archive/delete. iOS: URLRepositoryTests multiple archive/pending-delete state transitions. Future physical UI selection.</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -5550,27 +5550,27 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>SOURCE_CONFIRMED_WITH_DEVICE_GAP</t>
+          <t>LOCAL_PASS_WITH_DEVICE_UI_GAP</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>PASS(source): Android selectedEntryIds/EntrySelectionBar/archiveEntries/markPendingDeleteEntries確認。iOS EntrySelectionBar/archive(entryIDs)/markPendingDelete(entryIDs)確認。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.MainListViewModelTest 成功。PASS: xcodebuild test -only-testing:URLSaveriOSTests/URLRepositoryTests 成功、10 tests。</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>物理端末UI操作と専用UIテスト未実施。</t>
+          <t>物理端末UI操作は未検証。iOSは保存層の複数件状態遷移を検証済みだが、RootViewの選択バー操作そのものは未検証。</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>修正なし: 台帳未記載の既存機能として追加。</t>
+          <t>TESTED_LOCAL: Android ViewModel一括archive/pending deleteの成功/失敗混在をテスト追加。iOS URLRepositoryで複数件archive/pending delete状態遷移をテスト追加。</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>未実施: UI実操作確認が必要。</t>
+          <t>PASS local retest: Android MainListViewModelTest、iOS URLRepositoryTests 成功。物理UI選択/Undo操作は未実施。</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -5585,12 +5585,12 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>US-007/US-008の単体操作とは別の一括操作。</t>
+          <t>Batch selection local contract tests added 2026-06-29. UI operation still needs physical-device proof.</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>2026-06-29 00:49:24 +0900</t>
+          <t>2026-06-29 01:16:00 +0900</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore iOS collection parity flows
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -5065,27 +5065,27 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IOS_UI_GAP</t>
+          <t>LOCAL_PASS_WITH_DEVICE_UI_GAP</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>PASS: Android RepositoryBehaviorTest/MainListViewModelTest/ListFilterStateTest/TopFilterOrderResolutionTest対象実行成功。PASS: iOS URLRepositoryTests 12件成功、受信箱/作成/重複/移動/並び替え/削除時受信箱戻しを確認。</t>
+          <t>PASS: Android RepositoryBehaviorTest/MainListViewModelTest/ListFilterStateTest/TopFilterOrderResolutionTest対象実行成功。PASS: iOS URLRepositoryTests 12件成功、受信箱/作成/重複/移動/並び替え/削除時受信箱戻し/削除時同名ローカルタグ削除を確認。PASS: iOS ServiceFilterTests 18件成功、RootView/AppChrome/DetailViewのコレクション作成/選択/移動/削除/並び替え/検索/同名ローカルタグ込みフィルタ契約を確認。</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>iOSはcollectionsテーブル/API/URLRecord.collectionIDの土台を追加済み。自作コレクションの作成、移動、並び替え、フィルタUIは未実装。物理Androidで並び替え/削除は未検証。</t>
+          <t>物理Androidでコレクション並び替え/削除、物理iPhoneでコレクション作成/保存先選択/既存URL移動/削除/並び替え/フィルタUIは未検証。iOSの同名ローカルタグ連携は、詳細移動時の作成/割当、削除時の同名タグ削除、コレクション選択時の同名タグ付きURL表示までローカル実装済みだが、実機操作は未確認。</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>PARTIAL_FIXED_LOCAL: iOS collectionsテーブル、CollectionSummary、create/assign/reorder/delete/load API、collection_id DEFAULT 1を追加。US-035完全復元にはiOS UI接続が必要。</t>
+          <t>FIXED_LOCAL: iOS collectionsテーブル/API、AppModel.collections、上部コレクションチップ、+保存先作成、保存先管理シート、手動保存先選択、詳細画面の保存先表示/移動シート、削除/並び替え、同名ローカルタグ連携、検索/フィルタ連携を追加。Android同様に同名ローカルタグ付きURLも選択コレクションに含める。</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>PASS local retest: iOS URLRepositoryTests 12件成功。Android既存ローカルテストは前回成功済み。iOS UI実装/実機操作は未実施。</t>
+          <t>PASS local retest: iOS URLRepositoryTests + ServiceFilterTests 30件成功。Android既存ローカルテストは前回成功済み。iOS/Android物理UI操作は未実施。</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5095,17 +5095,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: コレクション作成/移動/並び替え/フィルタUIは未実装・未検証。</t>
+          <t>NOT VERIFIED on physical iPhone: コレクション作成/保存先選択/既存URL移動/削除/並び替え/フィルタUIは実機操作未検証。</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>iOS collection repository/API foundation added 2026-06-29; full UI parity still required.</t>
+          <t>iOS collection parity local implementation completed for create/filter/manual-save/detail-move/manage/delete/reorder/search/same-name local-tag linkage on 2026-06-29. Same-name local-tag filter parity added after gap audit. Physical-device proof still required.</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>2026-06-29 01:24:00 +0900</t>
+          <t>2026-06-29 01:43:21 +0900</t>
         </is>
       </c>
     </row>
@@ -5438,7 +5438,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>検索アイコンで検索欄を表示し、入力中はActive一覧が絞り込まれる。Androidはタイトル/URL/ホスト/コレクション名/割当ローカルタグ名、iOSはタイトル/URL/ホスト/割当ローカルタグ名を検索対象にする。未割当タグ名ではヒットしない。</t>
+          <t>検索アイコンで検索欄を表示し、入力中はActive一覧が絞り込まれる。Android/iOSともタイトル/URL/ホスト/コレクション名/割当ローカルタグ名を検索対象にする。未割当タグ名ではヒットしない。</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -5458,22 +5458,22 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.MainListViewModelTest 成功。PASS: xcodebuild test -only-testing:URLSaveriOSTests/ServiceFilterTests 成功、15 tests。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.MainListViewModelTest 成功。PASS: xcodebuild test -only-testing:URLSaveriOSTests/ServiceFilterTests 成功、17 tests。</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>物理Android/iPhoneでの検索欄表示、入力、クリア、戻る操作は未検証。iOSはcollections Repository/APIの土台は追加済みだが、RootView検索へのコレクション名連携はまだ未接続。</t>
+          <t>物理Android/iPhoneでの検索欄表示、入力、クリア、戻る操作は未検証。iOSのコレクション名検索はRootView/AppChrome経由で接続済みだが実機UI操作は未検証。</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>FIXED_LOCAL: Androidのタグ名検索が任意タグ名一致で全件ヒットし得る誤爆を修正。Android/iOSとも割当ローカルタグ名だけを検索対象にするテストを追加。</t>
+          <t>FIXED_LOCAL: Androidのタグ名検索が任意タグ名一致で全件ヒットし得る誤爆を修正。Android/iOSとも割当ローカルタグ名だけを検索対象にし、iOSもコレクション名検索を追加。</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>PASS local retest: Android MainListViewModelTest、iOS ServiceFilterTests 成功。UI実操作は未実施。</t>
+          <t>PASS local retest: Android MainListViewModelTest、iOS ServiceFilterTests 17件成功。UI実操作は未実施。</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -5483,17 +5483,17 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: 検索欄表示/入力/クリアは未検証。</t>
+          <t>NOT VERIFIED on physical iPhone: 検索欄表示/入力/クリアとコレクション名検索の実機操作は未検証。</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>User search local-tag false-positive fixed 2026-06-29. iOS collection repository/API foundation exists; collection-name search still needs RootView/UI wiring.</t>
+          <t>User search local-tag false-positive fixed 2026-06-29. iOS collection-name search wired and tested 2026-06-29.</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>2026-06-29 01:24:30 +0900</t>
+          <t>2026-06-29 01:32:41 +0900</t>
         </is>
       </c>
     </row>
@@ -5983,13 +5983,12 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6007,7 +6006,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ANDROID_LOCAL_PASS_WITH_IOS_MODEL_DIFFERENCE</t>
+          <t>DOCUMENTED_PASS_WITH_FINAL_SHA_GAP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6019,7 +6018,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DOCUMENTED_PASS_WITH_FINAL_SHA_GAP</t>
+          <t>FOUNDATION_ONLY_NOT_USER_FACING</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6031,48 +6030,48 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FOUNDATION_ONLY_NOT_USER_FACING</t>
+          <t>LOCAL_PASS: Web build/typecheck成功。本番DB/API実動作は未検証</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LOCAL_PASS: Web build/typecheck成功。本番DB/API実動作は未検証</t>
+          <t>LOCAL_PASS_WITH_DEPLOY_GAP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEPLOY_GAP</t>
+          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
+          <t>LOCAL_PASS_WITH_DEVICE_UI_GAP</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -6127,7 +6126,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_LIVE_GAP</t>
+          <t>LOCAL_PASS_WITH_UI_DEVICE_GAP</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6139,7 +6138,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_MAIL_GAP</t>
+          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_LIVE_GAP</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6151,19 +6150,19 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android実機PASS、iPhone UI操作は未検証</t>
+          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_MAIL_GAP</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android実機PASS、iPhone launchのみPASS</t>
+          <t>PARTIAL_PASS: Android実機PASS、iPhone UI操作は未検証</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6175,19 +6174,19 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS_WITH_LOCAL_DB_GAP</t>
+          <t>PARTIAL_PASS: Android実機PASS、iPhone launchのみPASS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS_WITH_SIMULATOR_WARNINGS</t>
+          <t>PARTIAL_PASS_WITH_CORE_SIMULATOR_WARNING</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6199,7 +6198,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PASS: Androidローカル検証成功、release buildも成功、実機共有系は未検証</t>
+          <t>PARTIAL_PASS_WITH_LOCAL_DB_GAP</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6211,7 +6210,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PASS: Web管理画面 typecheck/build 成功</t>
+          <t>PASS: Androidローカル検証成功、release buildも成功、実機共有系は未検証</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6223,7 +6222,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PASS: 正準スプレッドシート/CSV更新済み</t>
+          <t>PASS: Web管理画面 typecheck/build 成功</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -6235,7 +6234,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SOURCE_CONFIRMED_WITH_DEVICE_GAP</t>
+          <t>PASS: 正準スプレッドシート/CSV更新済み</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -6244,19 +6243,6 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>SOURCE_CONFIRMED_WITH_UI_TEST_GAP</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Align privacy disclosure and release verification
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'canonical_story_status'!$A$1:$S$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'canonical_story_status'!$A$1:$S$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,7 +449,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:S57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -4110,12 +4110,12 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>FIXED_LOCAL: XLSXの_FilterDatabase定義をA1:S57へ更新し、summaryシートもCSV最新ステータス集計と残ゲート集計から再生成。</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>PASS: CSV/XLSX更新後に行数/ID/XLSX dimension確認予定。</t>
+          <t>PASS: CSV 56行、XLSX dimension A1:S57、_FilterDatabase A1:S57、CSV/XLSXセル差分0、summaryステータス集計一致、summary残ゲート集計生成、XLSX zip integrity確認済み。</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -4130,12 +4130,12 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>US-034/US-035/US-036/AS-008/ES-006を追加。 US-037/US-038/US-039/US-040/TS-001を追加。 AS-009を追加し、US-039に公開reset-passwordページを追記。 US-006のiOS表示モード永続化ギャップを修正し、US-012にiOS BGTaskScheduler証跡を追記。 US-025/US-023/US-024のexport/entitlement近接テスト結果を更新。US-040にiOS PrivacyInfo証跡を補強。 iOS SharedTagCloud display_name migrationの冪等性を修正し、US-018/US-019/ES-003へ反映。</t>
+          <t>US-034/US-035/US-036/AS-008/ES-006を追加。 US-037/US-038/US-039/US-040/TS-001を追加。 AS-009を追加し、US-039に公開reset-passwordページを追記。 US-006のiOS表示モード永続化ギャップを修正し、US-012にiOS BGTaskScheduler証跡を追記。 US-025/US-023/US-024のexport/entitlement近接テスト結果を更新。US-040にiOS PrivacyInfo証跡を補強。 iOS SharedTagCloud display_name migrationの冪等性を修正し、US-018/US-019/ES-003へ反映。2026-06-29にXLSXフィルタ範囲、summaryステータス集計、残ゲート集計を実データへ修正。Public privacy stale検出後にsummary再生成。 Release privacy/store docsのpublic privacy stale反映後にsummary再生成。 Public web verifier追加後にsummary再生成。 Android privacy dialog文言更新後にsummary再生成。</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>2026-06-29 01:02:48 +0900</t>
+          <t>2026-06-29 02:11:30 +0900</t>
         </is>
       </c>
     </row>
@@ -4192,7 +4192,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>PASS: Androidローカル検証成功、release buildも成功、実機共有系は未検証</t>
+          <t>LOCAL_PASS_WITH_CONNECTED_TEST_GAP</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Release manifestで広告/AD_ID削除指定の対象なしwarning、MenuBook deprecated warningあり。どちらもbuild失敗ではない。物理共有/購入操作は未検証。</t>
+          <t>Release manifestで広告/AD_ID削除指定の対象なしwarning、MenuBook deprecated warningあり。どちらもbuild失敗ではない。connectedDebugAndroidTest、物理共有、購入操作は未検証。</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>PASS local retest。connectedDebugAndroidTestは実機データ保護のため未実施。</t>
+          <t>PASS local retest。connectedDebugAndroidTestは実機データ保護のため未実施。物理共有/購入操作は各ユーザーストーリー側で別ゲートとして追跡。</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -4227,12 +4227,12 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>connectedDebugAndroidTestは承認なし実行しない</t>
+          <t>connectedDebugAndroidTestは承認なし実行しない。2026-06-29にステータスをPASSからLOCAL_PASS_WITH_CONNECTED_TEST_GAPへ修正し、未検証ゲートを分離。</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>2026-06-29 00:39:51 +0900</t>
+          <t>2026-06-29 01:52:52 +0900</t>
         </is>
       </c>
     </row>
@@ -5331,7 +5331,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>web/invite-link/privacy/index.html; web/invite-link/account-deletion/index.html; web/invite-link/.well-known/assetlinks.json; web/invite-link/.well-known/apple-app-site-association; docs/release/final-submission-checklist.md</t>
+          <t>web/invite-link/privacy/index.html; web/invite-link/account-deletion/index.html; web/invite-link/.well-known/assetlinks.json; web/invite-link/.well-known/apple-app-site-association; scripts/verify_public_web_release.sh; docs/release/final-submission-checklist.md; docs/release/privacy-data-safety-draft.md; docs/release/store-listing-draft.md</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>docs/release/final-submission-checklist.md evidence; future: curl live URLs and JSON parse; store console values確認</t>
+          <t>scripts/verify_public_web_release.sh; docs/release/final-submission-checklist.md evidence; future: store console values確認</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -5356,27 +5356,27 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>DOCUMENTED_PASS_WITH_FINAL_SHA_GAP</t>
+          <t>PARTIAL_PUBLIC_PRIVACY_STALE_WITH_FINAL_SHA_GAP</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>PASS(documented): final-submission-checklistに2026-06-27 live URL 200/JSON parse証跡あり。Current turnではlive curl未再実行。</t>
+          <t>PARTIAL: 2026-06-29 live curlで privacy/account-deletion はHTTP 200、assetlinks.json/AASA はJSON parse成功。assetlinksは jp.miyamibu.urlalbum、AASAは 8R3B5675ZJ.com.mibu.codebridge.ios を含む。</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Play App Signing final SHA-256はNEEDS_USER_ACTION。今回ターンでは外部live URL再検証未実施。</t>
+          <t>BLOCKED_PUBLIC_DEPLOY_STALE: live privacy pageが「本物の課金も行いません」と表示し、repo sourceのStandard / Proサブスクリプション記述と不一致。Play App Signing final SHA-256もNEEDS_USER_ACTION。</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>修正なし: 台帳追跡行として追加。</t>
+          <t>FIXED_DOCS_LOCAL: final-submission-checklist、privacy-data-safety-draft、store-listing-draftを公開privacy staleとして更新。未修正: public privacy pageの再デプロイとfinal Play SHA-256差し替えが必要。</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>再テスト未実施: final SHA確定後にcurl/JSON parse/端末リンク確認が必要。</t>
+          <t>FAIL expected-current: scripts/verify_public_web_release.sh はHTTP/JSON/ID確認をPASSしつつ、privacyのStandard / Pro、Google Play Billing、StoreKit不足と stale no-real-billing文言2件を検出して5 issueで終了。再デプロイ後に同スクリプトを再実行する。</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5391,12 +5391,12 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>公開/ストア運用はコード機能ではないが、アプリ機能の到達性とストア審査に直結するためESとして追跡。</t>
+          <t>2026-06-29 live privacy staleを検出。repo source web/invite-link/privacy/index.html は課金あり文言に更新済みだが、miyamibu.xyz は古いno-real-billing文言を返す。privacy-data-safety-draft/store-listing-draftにも反映済み。scripts/verify_public_web_release.shで再検証可能。</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>2026-06-29 00:43:50 +0900</t>
+          <t>2026-06-29 02:08:03 +0900</t>
         </is>
       </c>
     </row>
@@ -5719,7 +5719,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>UrlSaverRoot.kt; strings.xml; AdsConfig.kt; AdsManager.kt; BannerAdSlot.kt; AdsConfigTest.kt; docs/release/final-submission-checklist.md; ios/URLSaveriOS/PrivacyInfo.xcprivacy; ios/URLSaverShareExtension/PrivacyInfo.xcprivacy</t>
+          <t>UrlSaverRoot.kt; strings.xml; AdsConfig.kt; AdsManager.kt; BannerAdSlot.kt; AdsConfigTest.kt; scripts/verify_public_web_release.sh; docs/release/final-submission-checklist.md; docs/release/privacy-data-safety-draft.md; docs/release/store-listing-draft.md; ios/URLSaveriOS/PrivacyInfo.xcprivacy; ios/URLSaverShareExtension/PrivacyInfo.xcprivacy</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -5734,7 +5734,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Android AdsConfigTest; source inspection for privacy dialog; release checklist review; future physical UI privacy dialog確認。</t>
+          <t>Android AdsConfigTest; source inspection for privacy dialog; scripts/verify_public_web_release.sh; release checklist review; future physical UI privacy dialog確認。</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -5744,27 +5744,27 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_STORE_DECLARATION_GAP</t>
+          <t>LOCAL_PASS_WITH_STORE_DECLARATION_AND_PUBLIC_PRIVACY_GAP</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew testDebugUnitTest --tests AdsConfigTest 成功。Source inspectionでprivacy_dialog stringsとUrlSaverRoot AlertDialogを確認。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.ads.AdsConfigTest 成功。PASS: ./gradlew assembleDebug 成功。Source inspectionでprivacy_dialog stringsとUrlSaverRoot AlertDialogを確認。</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>物理端末でのプライバシーダイアログ表示とPlay Console最終申告一致は未検証。</t>
+          <t>物理端末でのプライバシーダイアログ表示とPlay Console最終申告一致は未検証。2026-06-29時点のlive privacy pageは課金なし文言のままで、repo source/Standard-Pro課金復元と不一致。修正前のAndroidアプリ内privacy dialogも共有タグクラウド、問い合わせ、Standard/Pro購入を説明していなかった。</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>修正なし: 台帳未記載の既存ユーザー/ストア影響機能として追加。</t>
+          <t>PARTIAL_FIXED_LOCAL: Androidアプリ内privacy dialogを、端末内保存、メタデータ取得、共有タグクラウド、問い合わせ送信、Standard/Pro Google Play Billing、広告/分析/クラッシュ収集なしの文言へ更新。final-submission-checklist/privacy-data-safety-draft/store-listing-draftにpublic privacy staleを反映。未修正: public privacy page再デプロイ、store console最終申告一致、物理UI表示確認。</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>未実施: store申告最終確認が必要。</t>
+          <t>PASS local: ./gradlew assembleDebug 成功。PASS local: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.ads.AdsConfigTest 成功。NOTE: 最初の jp.mimac.urlsaver.AdsConfigTest 指定はテストフィルタ不一致で失敗し、正しい完全修飾名で再実行済み。FAIL expected-current: scripts/verify_public_web_release.sh がlive privacy課金文言staleを5 issueで検出。</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -5779,12 +5779,12 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>ES-006は公開Web/リンク。これはAndroidアプリ内表示と広告ガード。 targeted unit pass 2026-06-29. iOS privacy manifests included in release source review.</t>
+          <t>ES-006は公開Web/リンク。これはAndroidアプリ内表示と広告ガード。 Android app privacy dialog source updated 2026-06-29. iOS privacy manifests included in release source review; iOS同等のアプリ内privacy dialogは未確認。public privacy staleをUS-040にも連動記録し、release privacy/store docsとverify_public_web_release.shへ反映。</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>2026-06-29 01:00:20 +0900</t>
+          <t>2026-06-29 02:11:30 +0900</t>
         </is>
       </c>
     </row>
@@ -5846,22 +5846,22 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew testDebugUnitTest --tests MigrationDedupTest.migration_8_9_preservesExistingData_andCreatesUserLabels 成功。DAO/Entity/Repository/APIはsource確認、UI入口は未確認。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests MigrationDedupTest.migration_8_9_preservesExistingData_andCreatesUserLabels 成功。DAO/Entity/Repository/APIはsource確認。追加監査でAndroid UI/testsにUserLabel操作参照なし、iOSに同等UserLabelモデル/APIなし、git履歴上もdata foundation由来で旧UI削除ではないことを確認。</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>機能基礎はあるが現行ユーザーUI未実装。iOS側に同等UserLabelモデルは未確認。</t>
+          <t>機能基礎はあるが現行ユーザーUI未実装。iOS側にも同等UserLabelモデル/API/UIなし。旧UI復元対象ではなく、公開ユーザー機能にするなら新規仕様判断が必要。</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>未修正: 仕様化するならAndroid UI追加とiOS parity設計が必要。現状は未実装基盤として記録。</t>
+          <t>未修正: DESIGN.mdでadvanced taggingは明示承認なしに広げない方針。既存のローカルタグ/コレクションと重複するため、現状は未公開基盤として維持。</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>未実施: UI実装後に再テスト。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.MigrationDedupTest.migration_8_9_preservesExistingData_andCreatesUserLabels 成功。PASS audit: Android/iOS UI入口なしをrgで再確認。UI実装は未実施。</t>
         </is>
       </c>
       <c r="P56" t="inlineStr">
@@ -5876,12 +5876,12 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>ユーザー依頼の「基礎は作ったが実装していないもの」候補として追跡。 targeted unit pass 2026-06-29.</t>
+          <t>ユーザー依頼の「基礎は作ったが実装していないもの」候補として追跡。2026-06-29追加監査で旧実装UIの削除ではなくfoundation-onlyと判断。</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>2026-06-29 00:50:01 +0900</t>
+          <t>2026-06-29 01:49:20 +0900</t>
         </is>
       </c>
     </row>
@@ -5987,8 +5987,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6006,7 +6006,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DOCUMENTED_PASS_WITH_FINAL_SHA_GAP</t>
+          <t>FOUNDATION_ONLY_NOT_USER_FACING</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6018,24 +6018,24 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FOUNDATION_ONLY_NOT_USER_FACING</t>
+          <t>LOCAL_PASS: Web build/typecheck成功。本番DB/API実動作は未検証</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LOCAL_PASS: Web build/typecheck成功。本番DB/API実動作は未検証</t>
+          <t>LOCAL_PASS_WITH_CONNECTED_TEST_GAP</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6114,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_STORE_DECLARATION_GAP</t>
+          <t>LOCAL_PASS_WITH_STORE_DECLARATION_AND_PUBLIC_PRIVACY_GAP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6210,7 +6210,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PASS: Androidローカル検証成功、release buildも成功、実機共有系は未検証</t>
+          <t>PARTIAL_PUBLIC_PRIVACY_STALE_WITH_FINAL_SHA_GAP</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6240,6 +6240,142 @@
       <c r="B21" t="inlineStr">
         <is>
           <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>remaining_gate</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>story_ids</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>physical_Android</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>US-001,US-002,US-003,US-004,US-005,US-006,US-007,US-008,US-009,US-010,US-011,US-012,US-013,US-014,US-015,US-016,US-017,US-018,US-019,US-020,US-021,US-022,US-023,US-024,US-025,US-026,US-027,US-028,US-029,US-030,ES-002,US-031,US-032,US-033,US-034,US-035,US-036,US-037,US-038,US-039,US-040</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>physical_iPhone</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>US-001,US-002,US-003,US-004,US-005,US-006,US-007,US-008,US-009,US-010,US-011,US-012,US-013,US-014,US-015,US-016,US-017,US-018,US-019,US-020,US-021,US-022,US-023,US-024,US-025,US-026,US-027,US-028,US-029,US-030,ES-003,US-031,US-032,US-033,US-034,US-035,US-036,US-037,US-038,US-039</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>supabase_or_auth_live</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>US-016,US-018,US-019,US-023,US-024,AS-001,AS-002,AS-003,AS-004,AS-005,AS-006,ES-005,US-031,US-032,US-033,AS-007,US-036,AS-008,US-039</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>store_or_public_console</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>US-033,US-036,ES-006,US-040</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>public_privacy_deploy_stale</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ES-006,US-040</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>resend_live</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>AS-008,AS-009</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>connected_android_instrumentation</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ES-002</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore privacy flow and harden live gates
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -449,7 +449,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -608,7 +608,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2548,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3048,7 +3048,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3145,7 +3145,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3227,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3242,7 +3242,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -3324,7 +3324,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestは実機データ保護のため未実行。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>2026-06-27 15:51:33 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -4130,12 +4130,12 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>US-034/US-035/US-036/AS-008/ES-006を追加。 US-037/US-038/US-039/US-040/TS-001を追加。 AS-009を追加し、US-039に公開reset-passwordページを追記。 US-006のiOS表示モード永続化ギャップを修正し、US-012にiOS BGTaskScheduler証跡を追記。 US-025/US-023/US-024のexport/entitlement近接テスト結果を更新。US-040にiOS PrivacyInfo証跡を補強。 iOS SharedTagCloud display_name migrationの冪等性を修正し、US-018/US-019/ES-003へ反映。2026-06-29にXLSXフィルタ範囲、summaryステータス集計、残ゲート集計を実データへ修正。Public privacy stale検出後にsummary再生成。 Release privacy/store docsのpublic privacy stale反映後にsummary再生成。 Public web verifier追加後にsummary再生成。 Android privacy dialog文言更新後にsummary再生成。</t>
+          <t>US-034/US-035/US-036/AS-008/ES-006を追加。 US-037/US-038/US-039/US-040/TS-001を追加。 AS-009を追加し、US-039に公開reset-passwordページを追記。 US-006のiOS表示モード永続化ギャップを修正し、US-012にiOS BGTaskScheduler証跡を追記。 US-025/US-023/US-024のexport/entitlement近接テスト結果を更新。US-040にiOS PrivacyInfo証跡を補強。 iOS SharedTagCloud display_name migrationの冪等性を修正し、US-018/US-019/ES-003へ反映。2026-06-29にXLSXフィルタ範囲、summaryステータス集計、残ゲート集計を実データへ修正。Public privacy stale検出後にsummary再生成。 Release privacy/store docsのpublic privacy stale反映後にsummary再生成。 Public web verifier追加後にsummary再生成。 Android privacy dialog文言更新後にsummary再生成。 iOS PrivacyInfoSheet反映後にsummary再生成。 connectedDebugAndroidTest AVD PASS反映後にsummary再生成。</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>2026-06-29 02:11:30 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -4192,17 +4192,17 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_CONNECTED_TEST_GAP</t>
+          <t>PASS_WITH_PHYSICAL_OPERATION_GAP</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>PASS: 2026-06-29 ./gradlew assembleDebug testDebugUnitTest lintDebug 成功。PASS: ./gradlew assembleRelease 成功。対象追加確認として SharedTagAuthViewModelTest/TagRepositoryTest 単独実行も成功。</t>
+          <t>PASS: 2026-06-29 ./gradlew assembleDebug testDebugUnitTest lintDebug 成功。PASS: ./gradlew assembleRelease 成功。PASS: urlsaverParityApi35 AVDで connectedDebugAndroidTest 成功（17 tests、SharedTagCloudLiveDeviceTest 1件はlive Supabase設定なしでSKIP）。対象追加確認として SharedTagAuthViewModelTest/TagRepositoryTest 単独実行も成功。</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Release manifestで広告/AD_ID削除指定の対象なしwarning、MenuBook deprecated warningあり。どちらもbuild失敗ではない。connectedDebugAndroidTest、物理共有、購入操作は未検証。</t>
+          <t>Release manifestで広告/AD_ID削除指定の対象なしwarning、MenuBook deprecated warningあり。どちらもbuild失敗ではない。物理共有、購入操作は未検証。SharedTagCloudLiveDeviceTestはlive Supabase設定なしでSKIPし、Supabase/Auth live側に残す。</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>PASS local retest。connectedDebugAndroidTestは実機データ保護のため未実施。物理共有/購入操作は各ユーザーストーリー側で別ゲートとして追跡。</t>
+          <t>PASS local + connected retest。connectedDebugAndroidTestはテスト専用AVD urlsaverParityApi35で成功。物理共有/購入操作は各ユーザーストーリー側で別ゲートとして追跡。</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -4227,12 +4227,12 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>connectedDebugAndroidTestは承認なし実行しない。2026-06-29にステータスをPASSからLOCAL_PASS_WITH_CONNECTED_TEST_GAPへ修正し、未検証ゲートを分離。</t>
+          <t>connectedDebugAndroidTestは通常端末では承認なし実行しない。テスト専用AVDでは2026-06-29に実行済み。2026-06-29にステータスをPASSからLOCAL_PASS_WITH_CONNECTED_TEST_GAPへ修正し、未検証ゲートを分離。 2026-06-29 connectedDebugAndroidTestをテスト専用AVDで実行し成功。</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>2026-06-29 01:52:52 +0900</t>
+          <t>2026-06-29 06:32:51 +0900</t>
         </is>
       </c>
     </row>
@@ -4483,7 +4483,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS_WITH_LOCAL_DB_GAP</t>
+          <t>PASS_LINKED_DB_WITH_ADVISORY_WARNINGS</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -4493,17 +4493,17 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Supabase local DB/RLS live validationは未実施。ローカルPostgres 127.0.0.1:55422 が接続拒否。linked/prod DBは秘密値と明示承認なしで未接続。</t>
+          <t>linked DB schema/RPC validationは実施済み。残りはDB advisorsの既存WARN確認と、ローカルDB起動なしによりlocal lintが未実施である点。</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>APPLIED_LINKED_DB: 未適用だったshared group/profile、promo delivery inbox、contact support request、store purchase verification系schemaをlinked DBへ適用。PUBLIC実行権限が残っていたSECURITY DEFINER RPCをhardenし、anon実行は招待preview系だけに限定。</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>PASS Edge Function type check。DB lint/RLS/migration live testはローカルDB起動またはlinked DB承認後に再実行。</t>
+          <t>PASS linked DB: db query --linkedで主要table/RPC存在確認成功。PASS functions: contact-support/contact-support-resend-webhook/verify-store-purchase deploy成功。PASS advisors improvement: anon executable SECURITY DEFINERはpreview系3件のみ。Remaining advisors WARN: function search_path、signed-in SECURITY DEFINER、RLS initplan、multiple policies、leaked password protection。</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -4518,12 +4518,12 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t/>
+          <t>linked project xocumgxbylmpoobfqows。db pushはremote migration history driftにより不可だったため、必要migrationをdb query --linkedで個別適用。</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>2026-06-29 00:39:51 +0900</t>
+          <t>2026-06-29 07:25:00 +0900</t>
         </is>
       </c>
     </row>
@@ -4784,17 +4784,17 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Google Play sandbox purchase、StoreKit sandbox purchase、Edge Function deploy、migration適用、RTDN/App Store Server Notificationsは未検証。Supabase local db lintはローカルDB未起動で失敗。</t>
+          <t>Google Play sandbox purchase、StoreKit sandbox purchase、RTDN/App Store Server Notificationsは未検証。linked DB schemaとverify-store-purchase Function deployは確認済み。</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>実装済み: Store purchase verification table/migrationとEdge Functionを追加し、client purchase serviceから呼ぶ契約を整備。</t>
+          <t>実装済み: Store purchase verification table/migrationとEdge Functionを追加し、client purchase serviceから呼ぶ契約を整備。本番Function version 13へdeploy済み。</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>PASS local/type/build retest。外部ストアsandboxとSupabase deployは未実施。</t>
+          <t>PASS local/type/build retest。PASS linked DB: public.store_purchase_verifications と user_entitlement_grants 制約確認。PASS Function deploy/list: verify-store-purchase ACTIVE version 13。未実施: 外部ストアsandbox購入と通知。</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
@@ -4814,7 +4814,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>2026-06-29 00:39:51 +0900</t>
+          <t>2026-06-29 07:25:00 +0900</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEPLOY_GAP</t>
+          <t>PASS_LINKED_DB_WITH_STORE_WEBHOOK_GAP</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -4881,17 +4881,17 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>本番/linked DB migration適用、RLS live verification、失効webhookは未検証。ローカルDB未起動でSupabase lint不可。</t>
+          <t>ストア実通知、sandbox購入、管理画面からの実監査操作は未検証。linked DB migration/RLS/schema validationは実施済み。</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>実装済み: 検証履歴table、RLS、transaction unique index、grant作成処理を追加。</t>
+          <t>APPLIED_LINKED_DB: store purchase verification table/RLS/index、transaction unique index、grant作成処理をlinked DBへ適用。本番verify-store-purchase Functionもdeploy済み。</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>PASS local type/source retest。DB live validationは未実施。</t>
+          <t>PASS linked DB: store_purchase_verifications columns/RLS policy確認。PASS Function: verify-store-purchase no-session request is rejected with 401. Remaining: Google Play/App Store sandbox実取引と通知イベント。</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -4911,7 +4911,7 @@
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>2026-06-29 00:39:51 +0900</t>
+          <t>2026-06-29 07:25:00 +0900</t>
         </is>
       </c>
     </row>
@@ -5162,7 +5162,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_LIVE_GAP</t>
+          <t>LINKED_RPC_PASS_WITH_CHATGPT_CONSUMPTION_GAP</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -5172,7 +5172,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Supabase live RPC実行、ChatGPT側実消費、物理端末toggle操作は未検証。</t>
+          <t>ChatGPT側実消費と物理端末toggle操作は未検証。linked DB上のpersonal link table/RPC存在は確認済み。</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -5182,7 +5182,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>再テスト未実施: live Supabase環境が必要。</t>
+          <t>PASS linked DB: personal_link_sync_settings/personal_saved_links と set_personal_link_chatgpt_sync/apply_personal_link_ops RPC存在確認。Remaining: ChatGPT側実消費、サインイン済みユーザーによるtoggle実行。</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>2026-06-29 00:43:50 +0900</t>
+          <t>2026-06-29 07:25:00 +0900</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5259,7 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_RESEND_LIVE_GAP</t>
+          <t>PASS_RESEND_SENT_WITH_DELIVERY_EVENT_GAP</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -5269,17 +5269,17 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Resend live送信/配信/バウンスwebhook、Supabase DB live row確認は未検証。</t>
+          <t>Resend delivered/bounced/complained等の実webhookイベント反映は未確認。問い合わせ送信、Resend accepted相当のemail.sent、DB監査row、message id保存は確認済み。</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>修正なし: ローカル型/単体テスト上のエラー未検出。</t>
+          <t>FIXED_LIVE: contact-support-resend-webhookを本番deploy。contact-support Functionをpublic.contact_support_requests契約へ修正し、問い合わせ本文/メール/名前の原文を監査DBへ保存しない形へ変更。Resend message idを保存し、webhookが後続更新できる状態にした。</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>PASS local/type retest。live deliveryは未実施。</t>
+          <t>PASS live send: contact-support POST returned 202 accepted requestId=56d99d04-bbea-4b48-be13-eef62cb1f8d4。PASS DB: delivery_status=sent, delivery_provider=resend, has_message_id=true, delivery_event_type=email.sent。PASS webhook smoke: unsigned webhook returns 401 Invalid webhook secret。15秒後の確認ではdelivered webhook未反映。</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5294,12 +5294,12 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>US-022のユーザー問い合わせ導線に対応する管理/配信監査行。</t>
+          <t>Resend配送完了truthはResend側webhook実イベントまたはResend API照会が必要。</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>2026-06-29 00:43:50 +0900</t>
+          <t>2026-06-29 07:25:00 +0900</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>PARTIAL_PUBLIC_PRIVACY_STALE_WITH_FINAL_SHA_GAP</t>
+          <t>PASS_PUBLIC_WEB_WITH_FINAL_SHA_GAP</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -5366,17 +5366,17 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>BLOCKED_PUBLIC_DEPLOY_STALE: live privacy pageが「本物の課金も行いません」と表示し、repo sourceのStandard / Proサブスクリプション記述と不一致。Play App Signing final SHA-256もNEEDS_USER_ACTION。</t>
+          <t>Play App Signing final SHA-256はNEEDS_USER_ACTION。公開privacy staleは2026-06-29本番deploy後に解消済み。</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>FIXED_DOCS_LOCAL: final-submission-checklist、privacy-data-safety-draft、store-listing-draftを公開privacy staleとして更新。未修正: public privacy pageの再デプロイとfinal Play SHA-256差し替えが必要。</t>
+          <t>FIXED_PUBLIC_DEPLOY: web/invite-link をVercel project invite-linkへproduction deployし、miyamibu.xyzへalias済み。未修正: final Play SHA-256差し替えはGoogle Play Consoleの外部操作が必要。</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>FAIL expected-current: scripts/verify_public_web_release.sh はHTTP/JSON/ID確認をPASSしつつ、privacyのStandard / Pro、Google Play Billing、StoreKit不足と stale no-real-billing文言2件を検出して5 issueで終了。再デプロイ後に同スクリプトを再実行する。</t>
+          <t>PASS: npx --yes vercel@latest --prod --yes 成功。deployment dpl_8WZa3BBdqQs4f8s8mKcvxzaspVdv / alias https://miyamibu.xyz。PASS: scripts/verify_public_web_release.sh は privacy/account-deletion HTTP 200、assetlinks/AASA ID、Standard / Pro、Google Play Billing、StoreKit、stale no-real-billing文言なしを全て確認。</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5391,12 +5391,12 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>2026-06-29 live privacy staleを検出。repo source web/invite-link/privacy/index.html は課金あり文言に更新済みだが、miyamibu.xyz は古いno-real-billing文言を返す。privacy-data-safety-draft/store-listing-draftにも反映済み。scripts/verify_public_web_release.shで再検証可能。</t>
+          <t>2026-06-29 live privacy staleはproduction deployで解消。残りはPlay Console final SHA-256など外部Console確認のみ。</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>2026-06-29 02:08:03 +0900</t>
+          <t>2026-06-29 07:25:00 +0900</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Android/Store</t>
+          <t>Android/iOS/Store</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -5719,7 +5719,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>UrlSaverRoot.kt; strings.xml; AdsConfig.kt; AdsManager.kt; BannerAdSlot.kt; AdsConfigTest.kt; scripts/verify_public_web_release.sh; docs/release/final-submission-checklist.md; docs/release/privacy-data-safety-draft.md; docs/release/store-listing-draft.md; ios/URLSaveriOS/PrivacyInfo.xcprivacy; ios/URLSaverShareExtension/PrivacyInfo.xcprivacy</t>
+          <t>UrlSaverRoot.kt; strings.xml; AdsConfig.kt; AdsManager.kt; BannerAdSlot.kt; AdsConfigTest.kt; scripts/verify_public_web_release.sh; docs/release/final-submission-checklist.md; docs/release/privacy-data-safety-draft.md; docs/release/store-listing-draft.md; ios/URLSaveriOS/UI/RootView.swift; ios/URLSaveriOS/PrivacyInfo.xcprivacy; ios/URLSaverShareExtension/PrivacyInfo.xcprivacy</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -5729,12 +5729,12 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>プライバシーダイアログ文言が表示可能で、ADS_ENABLED/ADS_TRIAL_LAUNCH_ADS_ENABLEDが無効ならSDK初期化、バナー、インタースティシャルが走らない。</t>
+          <t>AndroidのプライバシーダイアログとiOSのデータ取り扱いシートが表示可能で、ADS_ENABLED/ADS_TRIAL_LAUNCH_ADS_ENABLEDが無効ならSDK初期化、バナー、インタースティシャルが走らない。</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Android AdsConfigTest; source inspection for privacy dialog; scripts/verify_public_web_release.sh; release checklist review; future physical UI privacy dialog確認。</t>
+          <t>Android AdsConfigTest; Android source inspection for privacy dialog; iOS source inspection/generic build for PrivacyInfoSheet; scripts/verify_public_web_release.sh; release checklist review; future physical UI privacy dialog/sheet確認。</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -5744,27 +5744,27 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_STORE_DECLARATION_AND_PUBLIC_PRIVACY_GAP</t>
+          <t>LOCAL_PASS_WITH_STORE_DECLARATION_GAP</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.ads.AdsConfigTest 成功。PASS: ./gradlew assembleDebug 成功。Source inspectionでprivacy_dialog stringsとUrlSaverRoot AlertDialogを確認。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.ads.AdsConfigTest 成功。PASS: ./gradlew assembleDebug 成功。PASS: xcodebuild -quiet -project ios/URLSaveriOS.xcodeproj -scheme URLSaveriOS -destination generic/platform=iOS Simulator CODE_SIGNING_ALLOWED=NO build 成功。Source inspectionでAndroid privacy_dialog strings/UrlSaverRoot AlertDialogとiOS RootView PrivacyInfoSheet/info.circle入口を確認。</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>物理端末でのプライバシーダイアログ表示とPlay Console最終申告一致は未検証。2026-06-29時点のlive privacy pageは課金なし文言のままで、repo source/Standard-Pro課金復元と不一致。修正前のAndroidアプリ内privacy dialogも共有タグクラウド、問い合わせ、Standard/Pro購入を説明していなかった。</t>
+          <t>物理端末でのAndroidプライバシーダイアログ/iOSデータ取り扱いシート表示とPlay Console/App Store最終申告一致は未検証。修正前のAndroidアプリ内privacy dialogは共有タグクラウド、問い合わせ、Standard/Pro購入を説明していなかった。修正前のiOSはPrivacyInfo.xcprivacyはあったが、アプリ内でユーザーが確認できる同等シートがなかった。live privacy pageの課金なし文言staleは2026-06-29本番deploy後に解消済み。</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>PARTIAL_FIXED_LOCAL: Androidアプリ内privacy dialogを、端末内保存、メタデータ取得、共有タグクラウド、問い合わせ送信、Standard/Pro Google Play Billing、広告/分析/クラッシュ収集なしの文言へ更新。final-submission-checklist/privacy-data-safety-draft/store-listing-draftにpublic privacy staleを反映。未修正: public privacy page再デプロイ、store console最終申告一致、物理UI表示確認。</t>
+          <t>PARTIAL_FIXED_LOCAL_AND_PUBLIC: Androidアプリ内privacy dialogを、端末内保存、メタデータ取得、共有タグクラウド、問い合わせ送信、Standard/Pro Google Play Billing、広告/分析/クラッシュ収集なしの文言へ更新。iOSはRootViewにinfo.circle入口とPrivacyInfoSheetを追加し、端末内保存、メタデータ取得、共有タグクラウド、問い合わせ、Standard/Pro StoreKit、広告/分析なしを表示。web/invite-link production deployでpublic privacy staleを解消。未修正: store console最終申告一致、物理UI表示確認。</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>PASS local: ./gradlew assembleDebug 成功。PASS local: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.ads.AdsConfigTest 成功。NOTE: 最初の jp.mimac.urlsaver.AdsConfigTest 指定はテストフィルタ不一致で失敗し、正しい完全修飾名で再実行済み。FAIL expected-current: scripts/verify_public_web_release.sh がlive privacy課金文言staleを5 issueで検出。</t>
+          <t>PASS local: ./gradlew assembleDebug 成功。PASS local: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.ads.AdsConfigTest 成功。PASS local: iOS generic simulator build成功。PASS public: scripts/verify_public_web_release.sh 成功。NOTE: 最初の jp.mimac.urlsaver.AdsConfigTest 指定はテストフィルタ不一致で失敗し、正しい完全修飾名で再実行済み。</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -5774,17 +5774,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t/>
+          <t>NOT VERIFIED on physical iPhone: データ取り扱いシート表示は実機操作未検証。</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>ES-006は公開Web/リンク。これはAndroidアプリ内表示と広告ガード。 Android app privacy dialog source updated 2026-06-29. iOS privacy manifests included in release source review; iOS同等のアプリ内privacy dialogは未確認。public privacy staleをUS-040にも連動記録し、release privacy/store docsとverify_public_web_release.shへ反映。</t>
+          <t>ES-006は公開Web/リンク。これはAndroid/iOSアプリ内表示と広告ガード。 Android app privacy dialog source updated 2026-06-29. iOS PrivacyInfoSheet/info.circle app UI added 2026-06-29 and generic build passed. public privacy staleはproduction deployで解消。</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>2026-06-29 02:11:30 +0900</t>
+          <t>2026-06-29 07:25:00 +0900</t>
         </is>
       </c>
     </row>
@@ -5983,12 +5983,14 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:S57"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C31"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6018,103 +6020,103 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LOCAL_PASS: Web build/typecheck成功。本番DB/API実動作は未検証</t>
+          <t>LINKED_RPC_PASS_WITH_CHATGPT_CONSUMPTION_GAP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_CONNECTED_TEST_GAP</t>
+          <t>LOCAL_PASS: Web build/typecheck成功。本番DB/API実動作は未検証</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEPLOY_GAP</t>
+          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
+          <t>LOCAL_PASS_WITH_DEVICE_UI_GAP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEVICE_UI_GAP</t>
+          <t>LOCAL_PASS_WITH_EXTERNAL_STORE_GAP</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_EXTERNAL_STORE_GAP</t>
+          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>19</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>LOCAL_PASS_WITH_RESEND_LIVE_GAP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_RESEND_LIVE_GAP</t>
+          <t>LOCAL_PASS_WITH_STORE_DECLARATION_GAP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_STORE_DECLARATION_AND_PUBLIC_PRIVACY_GAP</t>
+          <t>LOCAL_PASS_WITH_UI_DEVICE_GAP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6126,7 +6128,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_UI_DEVICE_GAP</t>
+          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_MAIL_GAP</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6138,55 +6140,55 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_LIVE_GAP</t>
+          <t>PARTIAL_PASS: Android実機PASS、iPhone UI操作は未検証</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_MAIL_GAP</t>
+          <t>PARTIAL_PASS: Android実機PASS、iPhone launchのみPASS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android実機PASS、iPhone UI操作は未検証</t>
+          <t>PARTIAL_PASS_WITH_CORE_SIMULATOR_WARNING</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android実機PASS、iPhone launchのみPASS</t>
+          <t>PASS: Web管理画面 typecheck/build 成功</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS_WITH_CORE_SIMULATOR_WARNING</t>
+          <t>PASS: 正準スプレッドシート/CSV更新済み</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6198,7 +6200,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS_WITH_LOCAL_DB_GAP</t>
+          <t>PASS_LINKED_DB_WITH_ADVISORY_WARNINGS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6210,7 +6212,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PARTIAL_PUBLIC_PRIVACY_STALE_WITH_FINAL_SHA_GAP</t>
+          <t>PASS_LINKED_DB_WITH_STORE_WEBHOOK_GAP</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6222,7 +6224,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PASS: Web管理画面 typecheck/build 成功</t>
+          <t>PASS_PUBLIC_WEB_WITH_FINAL_SHA_GAP</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -6234,7 +6236,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PASS: 正準スプレッドシート/CSV更新済み</t>
+          <t>PASS_RESEND_SENT_WITH_DELIVERY_EVENT_GAP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -6243,105 +6245,101 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>remaining_gate</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>story_ids</t>
-        </is>
-      </c>
-    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PASS_WITH_PHYSICAL_OPERATION_GAP</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>physical_Android</t>
+          <t>remaining_gate</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>count</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>US-001,US-002,US-003,US-004,US-005,US-006,US-007,US-008,US-009,US-010,US-011,US-012,US-013,US-014,US-015,US-016,US-017,US-018,US-019,US-020,US-021,US-022,US-023,US-024,US-025,US-026,US-027,US-028,US-029,US-030,ES-002,US-031,US-032,US-033,US-034,US-035,US-036,US-037,US-038,US-039,US-040</t>
+          <t>story_ids</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>physical_iPhone</t>
+          <t>physical_Android</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>36</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>US-001,US-002,US-003,US-004,US-005,US-006,US-007,US-008,US-009,US-010,US-011,US-012,US-013,US-014,US-015,US-016,US-017,US-018,US-019,US-020,US-021,US-022,US-023,US-024,US-025,US-026,US-027,US-028,US-029,US-030,ES-003,US-031,US-032,US-033,US-034,US-035,US-036,US-037,US-038,US-039</t>
+          <t>US-001,US-002,US-003,US-004,US-006,US-007,US-008,US-009,US-010,US-011,US-012,US-013,US-014,US-015,US-016,US-017,US-018,US-019,US-020,US-021,US-022,US-023,US-024,US-025,US-028,US-029,US-031,US-032,US-033,US-034,US-035,US-036,US-037,US-038,US-039,US-040</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>supabase_or_auth_live</t>
+          <t>physical_iPhone</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>41</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>US-016,US-018,US-019,US-023,US-024,AS-001,AS-002,AS-003,AS-004,AS-005,AS-006,ES-005,US-031,US-032,US-033,AS-007,US-036,AS-008,US-039</t>
+          <t>US-001,US-002,US-003,US-004,US-005,US-006,US-007,US-008,US-009,US-010,US-011,US-012,US-013,US-014,US-015,US-016,US-017,US-018,US-019,US-020,US-021,US-022,US-023,US-024,US-025,US-026,US-027,US-028,US-029,US-030,ES-003,US-031,US-032,US-033,US-034,US-035,US-036,US-037,US-038,US-039,US-040</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>store_or_public_console</t>
+          <t>supabase_or_auth_live</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>US-033,US-036,ES-006,US-040</t>
+          <t>US-016,US-018,US-019,US-023,US-024,US-031,US-032,US-039</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>public_privacy_deploy_stale</t>
+          <t>store_or_public_console</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ES-006,US-040</t>
+          <t>US-033,AS-007,ES-006,US-039,US-040,TS-001</t>
         </is>
       </c>
     </row>
@@ -6370,15 +6368,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ES-002</t>
+          <t/>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B30"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Align canonical identity and verification docs
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -1,63 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="canonical_story_status" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="stories" sheetId="1" r:id="rId1"/>
+    <sheet name="summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'canonical_story_status'!$A$1:$S$57</definedName>
-  </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="1">
     <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9EAF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9F2D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
-      </patternFill>
+      <patternFill patternType="none"/>
     </fill>
   </fills>
   <borders count="1">
@@ -72,96 +33,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -208,250 +82,24 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:latin typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
+      <a:fillStyleLst/>
+      <a:lnStyleLst/>
+      <a:effectStyleLst/>
+      <a:bgFillStyleLst/>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S57"/>
-  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -603,7 +251,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で手動貼り付け保存PASS、重複時挙動は未検証</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -628,22 +276,22 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PASS(Android physical Pixel 9a 55211JEBF16639): 一時URL https://example.com/rinbam-device-test-20260629-1214 を入力欄から保存し、一覧に example.com / 保存 12:15 / 自動取得できません が表示。証跡: artifacts/device-verification/2026-06-29/android-us001-add-form-ready-save.png, android-us001-after-save-final.png。</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 67fd5d37-d355-4a41-8f4a-c0949754bfce): 一時URL https://example.com/rinbam-iphone-device-test-20260629-1226 を入力欄から保存し、一覧に example.com / 保存 12:27 / 自動取得できません が表示。証跡: iphone-us001-add-form-filled.png, iphone-us001-after-save-final.png。</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t/>
+          <t>重複保存の実機挙動は次ループで別URL表記差分を使って確認する。既存ユーザーデータは削除/リセットしていない。</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 12:34:00 +0900</t>
         </is>
       </c>
     </row>
@@ -700,7 +348,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS_WITH_IPHONE_SHARE_EXTENSION_ERROR: Android実機の単一URL共有保存はPASS。iPhone実機は共有シートにりんばむ表示まで確認したが、選択後の保存引き継ぎが失敗。</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -710,37 +358,37 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>iPhone physical share extension: Safari共有シートで「りんばむ」を選択後、「アプリへ引き継げなかったため保存できませんでした」と表示。ShareViewControllerのhost app fallback/openHostApp経路または実機URL引き継ぎに問題の可能性。CoreSimulator/XCTest不整合は別件として継続。</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>未修正: US-002 iPhone共有拡張の保存引き継ぎ失敗を新規実機エラーとして記録。原因候補はShare Extensionからurlsaver://saveをopenするfallback経路、App Group repository初期化、または実機URL scheme引き継ぎ。</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
+          <t>Android physical retest PASS: ACTION_SEND text/plainで新規URLをShareReceiverActivityへ送り、「保存先タグ」シート -&gt; 「保存」 -&gt; 「保存しました」を確認。iPhone physical retest FAIL: Safari共有シートで「りんばむ」セルは表示されるが、選択後に保存できず失敗文言。connected Android instrumentationは2026-06-29 urlsaverParityApi35 AVDでPASS済み。</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PASS(Android physical Pixel 9a 55211JEBF16639, jp.miyamibu.urlalbum 1.0.13/13): ACTION_SEND text/plainで https://example.com/rinbam-us002-20260629125754 を共有。保存先タグシート、保存ボタン、保存後「保存しました」を確認。完了後ホームにexample.comカードが追加。証跡: android-us002-share-sheet.png/xml, android-us002-after-save.png/xml, android-us002-home-after-back.png/xml。</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>FAIL(iPhone physical 00008101-00066D96340A001E via Appium/WDA): Safariで https://example.com/rinbam-us002-ios-20260629130000 を開き、共有メニュー -&gt; 共有シートで「りんばむ」セルを確認。XCUIElementTypeCell label=りんばむ をクリック後、「アプリへ引き継げなかったため保存できませんでした」と表示。証跡: iphone-us002-safari.png/xml, iphone-us002-safari-more-menu.png/xml, iphone-us002-share-sheet.png/xml, iphone-us002-share-sheet-scroll-3.png/xml, iphone-us002-after-rinbam-element-click.png/xml。</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t/>
+          <t>iPhone共有シート上の表示名は「りんばむ」で旧名ではない。US-002完全PASSにはiPhone Share Extension保存成功または直接保存経路の修正と再テストが必要。</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 13:06:00 +0900</t>
         </is>
       </c>
     </row>
@@ -797,7 +445,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS_WITH_IPHONE_INPUT_GAP: Android実機の複数URL共有保存はPASS。iPhone実機は複数URL共有入力を生成できず、実保存未検証。</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -807,37 +455,37 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>iPhone physical US-003 input gap: Safari通常共有は単一URLのみ。Web Share APIで複数URLテキスト共有を作る一時ページを試したが、物理iPhone Safari上で navigator.share is not a function となり共有シートを生成できなかった。US-002では共有シートの「りんばむ」選択後に保存引き継ぎ失敗も確認済み。</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>未修正: US-003 iPhone複数URL共有の実機入力手段と、US-002で見つかったShare Extension保存引き継ぎ失敗の修正が必要。Android側の今回検証ではロジスティカル/UXエラーなし。</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
+          <t>Android physical retest PASS: ACTION_SEND_MULTIPLE + 改行区切りEXTRA_TEXTで新規2件をShareReceiverActivityへ送り、「保存先タグ」シート -&gt; 「保存」 -&gt; 「2件を処理しました（新規2 / 既存0 / 復元0 / 失敗0）」を確認。iPhone physical retest NOT VERIFIED for multi URL save: Web Share代替はnavigator.share未対応で共有シート生成不可。</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PASS(Android physical Pixel 9a 55211JEBF16639, jp.miyamibu.urlalbum 1.0.13/13): ACTION_SEND_MULTIPLE text/plainで https://example.com/rinbam-us003-a2-202606291309 と https://example.com/rinbam-us003-b2-202606291309 を改行区切りEXTRA_TEXTとして共有。保存先タグシート、保存ボタン、保存後「2件を処理しました（新規2 / 既存0 / 復元0 / 失敗0）」を確認。証跡: android-us003-share-sheet-retry.png/xml, android-us003-after-save.png/xml。</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>NOT VERIFIED on physical iPhone for US-003 multi URL save (00008101-00066D96340A001E via Appium/WDA): Safari通常共有は単一URLのみのためUS-003条件を満たさず。ローカル一時ページからWeb Share APIで複数URLテキスト共有を試したが、物理iPhone Safariで「navigator.share is not a function」と表示され共有シートを生成できなかった。証跡: iphone-us003-webshare-start.png/xml, iphone-us003-webshare-after-button.png/xml, us003-webshare/index.html。</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t/>
+          <t>Android投入時、adb --esa配列形式では実機am経由でURL抽出できず「URLが見つかりませんでした」になったため、テストで許容されるACTION_SEND_MULTIPLE + 改行区切りEXTRA_TEXTで再検証しPASS。iPhone US-003完全確認にはNotes/Files等から複数URLテキストを共有する実機手段、またはUS-002 Share Extension引き継ぎ修正後の再テストが必要。</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 13:11:27 +0900</t>
         </is>
       </c>
     </row>
@@ -894,47 +542,47 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS_WITH_NORMALIZATION_AND_IPHONE_UX_GAP: 両実機で同一URL重複は確認済み。表記違い正規化とiPhone通知導線は未完了。</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。 / PASS device partial: 2026-06-29 両実機で同一URLの重複保存を追加確認。</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>PARTIAL_DEVICE_GAP: Android/iPhone実機で同一URL重複判定は確認。表記違いURLの正規化重複は未検証。iPhone手動追加の重複保存後、コード上は「このURLはすでに保存済みです」+「見る」通知を5秒表示する設計だが、Appium証跡では保存後ホームに戻り通知が見えなかった。</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>未修正: 今回は検証結果の記録のみ。iPhone重複通知/見る導線はUX差分候補として次ループで原因特定と修正対象判定が必要。</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。 / RETEST NEEDED: 表記違い正規化、iPhone重複通知「見る」、修正後の両実機再確認。</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PARTIAL_PASS(Android physical Pixel 9a 55211JEBF16639): 既存URL https://example.com/rinbam-device-test-20260629-1214 をACTION_SENDでShareReceiverActivityへ渡し、保存押下後に「このURLはすでに保存されています」表示を確認。証跡: artifacts/device-verification/2026-06-29/android-us004-share-duplicate-before.png/xml, android-us004-share-duplicate-after.png/xml, android-us004-share-duplicate-result.png/xml。表記違い正規化重複は未検証。</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PARTIAL_PASS_WITH_UX_GAP(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8ea12d85-7105-48c3-ac0c-4b2b77650cf2): 既存URL https://example.com/rinbam-iphone-device-test-20260629-1226 を手動追加し、保存後にホームへ戻り既存1件表示のまま追加重複は見えなかった。証跡: iphone-us004-duplicate-before.png/xml, iphone-us004-duplicate-add-form.png/xml, iphone-us004-duplicate-filled.png/xml, iphone-us004-duplicate-result-after-save.png/xml。期待される「このURLはすでに保存済みです」+「見る」通知は証跡上未確認。表記違い正規化重複は未検証。</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t/>
+          <t>US-004は完全PASSではない。同一URL重複は両実機で進捗あり。残: 表記違いURLのnormalizedUrl重複、Android手動追加側の「見る」導線、iPhone通知/見る導線の表示確認または修正。</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 12:46:10 +0900</t>
         </is>
       </c>
     </row>
@@ -991,7 +639,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS: Android実機PASS、iPhoneホーム/フィルター表示PASS、保存URL絞り込み操作未実施</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1021,17 +669,17 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8eb5a3bf-b1a1-4d77-85ce-b691a9b44192): アプリ名「りんばむ」、ホーム表示、サービス/タグ系フィルタチップ、下部5アクションをXML/PNGで確認。証跡: artifacts/device-verification/2026-06-29/iphone-appium-home-after-rename.png, iphone-appium-home-source-after-rename.xml。保存済みURLを用いた絞り込み操作は未実施。</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t/>
+          <t>iPhone Appium/WDAが復旧しホーム表示証跡を取得。データ作成を伴うURL一覧/絞り込み操作は次ループで非破壊手順を設計して確認する。</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 11:48:00 +0900</t>
         </is>
       </c>
     </row>
@@ -1088,7 +736,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で表示モード切替PASS、再起動後保持は未検証</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1113,22 +761,22 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PASS(Android physical Pixel 9a 55211JEBF16639): 表示モードボタンをタップし content-desc が「画像つき表示へ切り替える」へ変化。証跡: artifacts/device-verification/2026-06-29/android-pixel9a-display-toggle-after.png, android-pixel9a-display-toggle-after.xml。</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8c957f69-e6f0-412a-9d20-816728e11a1b): 表示モードボタンをタップし、XMLで「画像なし表示へ切り替える」を確認。証跡: artifacts/device-verification/2026-06-29/iphone-ui-loop-display-toggle-after.png, iphone-ui-loop-display-toggle-after.xml。</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>iOS display mode persistence fixed 2026-06-29.</t>
+          <t>物理端末で切替自体は確認済み。再起動後保持、Archive/Tag detail反映は次ループで確認が必要。</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>2026-06-29 00:57:14 +0900</t>
+          <t>2026-06-29 12:03:48 +0900</t>
         </is>
       </c>
     </row>
@@ -1185,7 +833,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で詳細からアーカイブ/復元PASS、スワイプ操作とUndo実行は未検証</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1210,22 +858,22 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PARTIAL(Android physical Pixel 9a 55211JEBF16639): 詳細のアーカイブでactive一覧から消え、アーカイブ詳細でアーカイブ解除、active一覧へ復元。Undo表示は確認したが実行成功は未証明。証跡: android-us007-archive-after-tap.png, android-us007-archive-detail-open.png, android-us007-unarchive-after-tap.png。</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PARTIAL(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 67fd5d37-d355-4a41-8f4a-c0949754bfce): 詳細のアーカイブでactive一覧から消え、アーカイブ一覧に移動、アーカイブ済み詳細で削除無効/アーカイブ解除、active一覧へ復元。スワイプ/Undo実行は未証明。証跡: iphone-us007-archive-after-tap.png, iphone-us007-archive-list.png, iphone-us007-archive-detail.png, iphone-us007-unarchive-home.png。</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t/>
+          <t>この行の受入条件に含まれるスワイプ操作とUndo復帰は未完了。次ループで一時データを使い、猶予中Undoをタイミング込みで確認する。</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 12:34:00 +0900</t>
         </is>
       </c>
     </row>
@@ -1282,47 +930,47 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PHYSICAL_PASS_WITH_TEMP_DATA: 両実機で一時URLを使い、削除確認、5秒Undo通知、Undo後の一覧復帰を確認。</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: 既存のローカル/ビルド検証に加え、2026-06-29に両実機で一時URLを使った削除猶予/Undo導線を確認。</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>過去試行ではAndroidの座標タップが5秒Undoに間に合わず復元未証明だったが、今回bounds由来のUndo中心タップで復元を確認。iPhoneもAppium/WDA連続操作で復元確認。製品ロジック上の不具合は今回未検出。</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>修正対象なし: 実機再検証で削除猶予/Undoの期待動作を確認。</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
+          <t>PASS physical retest: Android Pixel 9a と iPhone 12 で削除確認文言、削除後通知「削除しました」「元に戻す」、Undo後のカード復帰を確認。</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PASS(Android physical Pixel 9a 55211JEBF16639, jp.miyamibu.urlalbum): 一時カード(保存 14:55/14:56系)で詳細削除確認「このURLは削除待ちに移動します。5秒以内なら元に戻せます。」、削除後Snackbar「削除しました」「元に戻す」、Undo後に一覧へ「保存 14:56」「保存 14:55」が復帰/残存することを確認。証跡: artifacts/device-verification/2026-06-29/us008/android-us008-delete-dialog-retry.*, android-us008-after-delete-retry.*, android-us008-after-undo-retry.*</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E, Appium/WDA, com.mibu.codebridge.ios): 一時URL https://example.com/rinbam-us008-iphone-202606291501 を追加し、詳細削除確認、削除後通知「削除しました」「元に戻す」、Undo後に「保存 15:03」のカードが一覧復帰することを確認。証跡: artifacts/device-verification/2026-06-29/us008/iphone-us008-temp-*.xml/png</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>通常端末の既存データは消さない</t>
+          <t>通常端末の既存データは消さず、一時テストURLのみ使用。iPhoneはAppium/WDA、AndroidはADB/uiautomator/screencapで証跡取得。</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 15:07:47 +0900</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1027,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で詳細遷移と外部で開く導線表示PASS、外部ブラウザ起動は未実行</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1404,22 +1052,22 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PARTIAL(Android physical Pixel 9a 55211JEBF16639): 一覧カードタップで詳細へ遷移し、開く/コピー/アーカイブ/削除/メモ編集/metadata失敗表示を確認。外部ブラウザ起動は未実行。証跡: android-us009-detail-open.png。</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PARTIAL(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 67fd5d37-d355-4a41-8f4a-c0949754bfce): 一覧カードタップで詳細へ遷移し、開く/コピー/アーカイブ/削除/メモ編集/metadata失敗表示を確認。外部ブラウザ起動は未実行。証跡: iphone-us009-detail-open.png。</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t/>
+          <t>外部ブラウザ起動は別アプリ遷移を伴うため未実行。次ループで戻り動作も含めて確認する。</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 12:34:00 +0900</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1124,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS: Android/iPhone実機でタイトル編集保存PASS、Undo実行は未検証</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1501,22 +1149,22 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PARTIAL(Android physical Pixel 9a 55211JEBF16639): タイトル編集UIを開き Rinbam Device Title を保存、詳細に反映。Undo表示は確認したが実行は未証明。証跡: android-us010-title-edit-open.png, android-us010-title-saved.png。</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PARTIAL(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 67fd5d37-d355-4a41-8f4a-c0949754bfce): タイトル編集UIを開き Rinbam iPhone Title を保存、詳細に反映。Undo通知は取得時点で確認できず、Undo実行は未証明。証跡: iphone-us010-title-edit-open.png, iphone-us010-title-saved.png。</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t/>
+          <t>タイトルUndoは次ループで保存直後に通知捕捉と実行確認を行う。</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 12:34:00 +0900</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1221,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PASS: Android/iPhone実機でメモ編集保存PASS</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1598,22 +1246,22 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PASS(Android physical Pixel 9a 55211JEBF16639): メモ編集UIを開き Android device memo 1216 を保存、詳細に反映。証跡: android-us011-memo-edit-open.png, android-us011-memo-saved.png。</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 67fd5d37-d355-4a41-8f4a-c0949754bfce): メモ編集ダイアログを開き iPhone device memo 1228 を保存、詳細に反映。証跡: iphone-us011-memo-edit-open.png, iphone-us011-memo-saved.png。</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t/>
+          <t>一時URLのメモ保存のみ確認。既存ユーザーデータは削除/リセットしていない。</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 12:34:00 +0900</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1318,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
+          <t>PARTIAL_PASS: Android/iPhone実機でmetadata失敗状態表示PASS、成功取得は未検証</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1695,22 +1343,22 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PARTIAL(Android physical Pixel 9a 55211JEBF16639): example.com 一時URLで一覧/詳細に 自動取得できません と HTTP_404 系説明、再取得導線表示を確認。成功取得は未検証。証跡: android-us001-after-save-final.png, android-us009-detail-open.png。</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PARTIAL(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 67fd5d37-d355-4a41-8f4a-c0949754bfce): example.com 一時URLで一覧/詳細に 自動取得できません、ページが見つかりませんでした (HTTP_404)、再取得導線表示を確認。成功取得は未検証。証跡: iphone-us001-after-save-final.png, iphone-us009-detail-open.png。</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>iOS BGTaskScheduler/BackgroundTaskRunner coverage added 2026-06-29.</t>
+          <t>iOS BGTaskScheduler/BackgroundTaskRunner coverage added 2026-06-29. 実機では失敗状態表示のみ確認。成功取得と再取得実行はUS-013側で継続確認する。</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>2026-06-29 00:57:14 +0900</t>
+          <t>2026-06-29 12:34:00 +0900</t>
         </is>
       </c>
     </row>
@@ -1767,47 +1415,47 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS_WITH_INTERNAL_CONTRACT_GAP: 両実機で失敗metadataの再取得UI導線と押下を確認。再enqueue/updatedAt不変は未検証。</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。</t>
+          <t>PASS: ./gradlew assembleDebug testDebugUnitTest lintDebug assembleRelease 成功。connectedDebugAndroidTestはurlsaverParityApi35 AVDでPASS。 / PARTIAL: iOS Release generic build と build-for-testing 成功。XCTest実行はCoreSimulator不整合で未実施。 / PASS device partial: 2026-06-29 Android/iPhone実機で失敗metadata詳細と再取得ボタン表示、押下操作を確認。</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>PARTIAL_DEVICE_GAP: 両実機で「再取得」ボタン表示と押下は確認。example.comのHTTP_404/ページ未検出状態のため、成功metadata取得は未確認。UI証跡だけでは再enqueue実行、WorkManager/MetadataCoordinator処理、metadata更新だけでupdatedAtを変えない契約は証明できない。</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>未修正: 今回は実機導線の確認と未検証内部契約の記録のみ。UI上の明確なクラッシュ/操作不能は未検出。必要ならログ/DB観測付きの非破壊検証を追加する。</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
+          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。 / RETEST NEEDED: 成功取得可能URLでのmetadata更新、再enqueueログ/DB観測、updatedAt不変確認。</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PARTIAL_PASS(Android physical Pixel 9a 55211JEBF16639): 既存URL詳細で「このURLは自動取得できません」「ページが見つからないため、自動取得できませんでした。」と「再取得」ボタンを確認し、再取得をタップ。短時間後も同じ404失敗表示。証跡: artifacts/device-verification/2026-06-29/android-us013-detail-before-retry.png/xml, android-us013-after-retry-tap.png/xml, android-us013-after-retry-settled.xml。再enqueue/updatedAt不変は未検証。</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PARTIAL_PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session c5da0df9-c429-41d4-acc2-c82b0575b95c): 既存URL詳細で「このURLは自動取得できません」「ページが見つかりませんでした (HTTP_404)」と「再取得」ボタンを確認し、再取得をタップ。短時間後も同じ404失敗表示。証跡: iphone-us013-detail-before-retry.png/xml, iphone-us013-after-retry-tap.png/xml, iphone-us013-after-retry-settled.xml。再enqueue/updatedAt不変は未検証。</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t/>
+          <t>US-013は実機UI導線の確認は前進。完全PASSには、成功取得可能URLまたはDB/ログ観測で再enqueueとupdatedAt不変を確認する必要がある。</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 12:52:04 +0900</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1512,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS_WITH_TAG_DELETE_AND_DUPLICATE_GAP: 両実機でローカルタグ作成とURLへの割当は確認。削除時関連付け解除、重複処理、タグ別件数は未確認。</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1874,37 +1522,37 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>未完了範囲: タグ削除時の関連付け解除、重複タグ名/既割当時の文言、タグ別URL件数表示は今回未確認。iPhoneではタグ追加後にキーボード表示中のシートを閉じる操作がAppiumで安定せず、詳細画面へ戻した後の表示確認は未完了。</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>修正対象未確定: Android/iPhoneともローカルタグ作成・割当の実機導線は動作。iPhoneのタグ編集シート閉じ操作は追加調査対象。削除/重複/件数表示は次回以降の検証対象。</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
+          <t>Android physical retest PARTIAL_PASS: 詳細タグ欄 -&gt; 編集 -&gt; 新しいタグ -&gt; タグを作成して追加で、現在のタグと詳細タグ欄に作成タグが表示。iPhone physical retest PARTIAL_PASS: 詳細タグ欄 -&gt; 編集 -&gt; 新しいタグ -&gt; タグを作成して追加で、現在のタグに us014-ios-1314 が表示。削除/重複/件数表示は未実施。</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PARTIAL_PASS(Android physical Pixel 9a 55211JEBF16639, jp.miyamibu.urlalbum 1.0.13/13): 既存URL詳細でタグ欄「まだタグは付いていません」と編集ボタンを確認。タグ編集シートで新規タグを作成して追加し、「現在のタグ」に作成タグが表示、閉じた後の詳細タグ欄にも表示を確認。証跡: android-us014-detail-start.png/xml, android-us014-tag-editor-open.png/xml, android-us014-tag-name-entered.png/xml, android-us014-after-create-assign.png/xml, android-us014-detail-after-tag.png/xml。削除/重複/件数表示は未確認。</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PARTIAL_PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 31809d80-ed0b-4331-8c1f-fc32cc1ad527): 既存URL詳細でタグ欄「まだタグは付いていません」とローカルタグ編集ボタンを確認。タグ編集シートで us014-ios-1314 を入力し「タグを作成して追加」を実行、「現在のタグ」に us014-ios-1314 と「外す」が表示。証跡: iphone-us014-detail-tags-visible.png/xml, iphone-us014-tag-editor-open.png/xml, iphone-us014-tag-name-entered.png/xml, iphone-us014-after-create-assign.png/xml。キーボード表示中のシート閉じ/詳細戻り表示、削除/重複/件数表示は未確認。</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t/>
+          <t>Androidは端末キーボード変換により入力タグ名が全角混じりになったが、作成・割当・詳細表示は確認済み。US-014完全PASSには、両実機で重複タグ名/既割当時の文言、タグ削除時の関連付け解除、タグ管理/タグ詳細でURL件数表示を確認する必要がある。</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 13:18:39 +0900</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1609,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PHYSICAL_PASS_WITH_ANDROID_LOCAL_TAG_COPY_UX_GAP: 両実機でタグ選択/タグ詳細から対象URLだけの一覧と詳細遷移を確認。Androidローカルタグ詳細の共有タグ文言はUX不整合。</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1971,37 +1619,37 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>Android UX: ローカルタグ詳細でも「クラウド共有を使うにはサインインが必要です」「この共有タグを削除」など共有タグ文言が表示される。iPhoneはタグチップ選択で対象URL1件に絞り込みできるが、独立したタグ詳細画面ではなくホーム一覧フィルタとして実装されている。</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>未修正: Androidのローカルタグ詳細文言をローカルタグ向けに分岐する改善候補。iPhoneは現行設計上フィルタ導線で機能達成。</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
+          <t>Android physical PASS: DB読取で tagId=1/entryId=4 の割当を確認後、urlsaver://tag/1 でタグ詳細を開き、タグ名、1件表示、対象URLカード、カードから詳細遷移を確認。iPhone physical PASS: Appium/WDAで us014-ios-1314 チップを横スクロール後にタップし、表示URLが2件から対象1件へ絞り込まれ、カードから詳細へ遷移することを確認。</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PASS on physical Android Pixel 9a 55211JEBF16639: artifacts/device-verification/2026-06-29/us015/android-us015-tag-detail.xml/png と android-us015-tag-detail-open-entry.xml/png。</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PASS on physical iPhone 12 UDID 00008101-00066D96340A001E via Appium/WDA: artifacts/device-verification/2026-06-29/us015/iphone-us015-after-tag-tap-source.json と iphone-us015-tag-open-entry-source.json。</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t/>
+          <t>非破壊確認のみ。Android DBは run-as で url_saver.db/-wal/-shm を読み取りコピーし、タグ割当を現在状態として照合。iPhoneはAppium session 2a3a89b1-ee18-4c91-8099-a11a7b00dbbf。</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 13:27:31 +0900</t>
         </is>
       </c>
     </row>
@@ -2145,7 +1793,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Android: MainActivityViewModelSecondaryIntentTest/ShareReceiverActivityEntrypointTest; iOS: PendingInviteStoreTests/URLSaverAppModel source + live tests</t>
+          <t>Android実機: adb am start deep link + uiautomator/screencap; iPhone実機: devicectl --payload-url + Appium/WDA source/screenshot; 既存unit/build結果参照</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2155,7 +1803,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PHYSICAL_PARTIAL_PASS_WITH_INVITE_UX_GAPS: 両実機で urlsaver://invite と https://miyamibu.xyz/invite が招待確認導線へ入ることを確認。Android HTTPSはローディング継続、iPhoneはraw error露出。実招待作成/参加は未検証。</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2165,37 +1813,37 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>iOS XCTest/UI操作: CoreSimulator不整合またはAppium RemoteXPC tunnel未起動により未完了。</t>
+          <t>Android HTTPS invite: 30秒以上「招待リンクを確認しています」から進まず、無効/失敗状態へ遷移しない。iPhone invalid invite: 「invalid_or_expired_invite」のraw errorが画面に露出し日本語UXになっていない。実招待作成/acceptは未検証。</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>修正対象なし: 環境/外部接続ブロックまたは未検証。コードのロジスティカル/UXエラーは今回の検証では未検出。</t>
+          <t>未修正: 今回は検証・記録のみ。修正候補はAndroid invite previewのタイムアウト/失敗表示、iOS remote errorの日本語マッピング。</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>再テスト未実施: 修正なし。ブロック解除後に再実行。 PASS connected Android instrumentation: 2026-06-29 urlsaverParityApi35 AVDで URLSAVER_ALLOW_CONNECTED_ANDROID_TESTS=true URLSAVER_APPROVE_ANDROID_APP_DATA_RESET=true ./gradlew connectedDebugAndroidTest 成功。</t>
+          <t>今回の再検証: Android physical Pixel 9aで urlsaver://invite は無効表示PASS、https inviteはローディング継続FAIL。iPhone physical + Appium/WDAで両形式とも招待確認画面遷移PASS、invalid raw error表示UX_FAIL。</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PHYSICAL_PARTIAL: Pixel 9a 55211JEBF16639 / jp.miyamibu.urlalbum v1.0.13。urlsaver://invite/codex-invalid-us017-20260629 は「招待リンクが無効か期限切れです」表示。https://miyamibu.xyz/invite/codex-invalid-us017-https-20260629 は招待確認画面へ入るが30秒以上ローディング継続。証跡: artifacts/device-verification/2026-06-29/us017/android-us017-*.png/xml</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PHYSICAL_PARTIAL: iPhone 12 UDID 00008101-00066D96340A001E / com.mibu.codebridge.ios v1.0.11 / Appium WDA session 1bf0b8f3-5c1a-49c8-8bf3-8f672e3ea7b0。urlsaver://invite と https://miyamibu.xyz/invite は招待確認画面へ遷移。無効時に「招待リンクを確認できませんでした」+ raw `invalid_or_expired_invite` 表示。証跡: artifacts/device-verification/2026-06-29/us017/iphone-us017-*.png/json</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t/>
+          <t>US-017はDeep Link受信/画面遷移は両実機で確認済み。実際の有効招待作成・参加・権限同期はSupabase liveユーザー状態が必要なため未完了。</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 14:49:26 +0900</t>
         </is>
       </c>
     </row>
@@ -2446,7 +2094,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で認証関連画面表示PASS、OAuth/サインアウト実行は未検証</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2471,22 +2119,22 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PASS/PARTIAL(Android physical Pixel 9a 55211JEBF16639): プロフィール画面で「Googleで続ける」「サインイン後に利用できます」を確認。実OAuthは未実施。証跡: android-pixel9a-profile-open-portrait.png/xml。</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PASS/PARTIAL(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8c957f69-e6f0-412a-9d20-816728e11a1b): プロフィールシートでアカウント表示、ChatGPT連携トグル、サインアウトボタンを確認。サインアウト/OAuth callbackは未実施。証跡: iphone-ui-loop-profile-open.png/xml, iphone-ui-loop-after-inquiry-close-correct.png/xml。</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>秘密値入力はユーザー操作のみ</t>
+          <t>秘密情報入力や外部OAuthは実行せず、画面表示のみ確認。</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 12:03:48 +0900</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2191,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS: Android/iPhone実機でプロフィール編集画面表示PASS、編集保存は未検証</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2568,22 +2216,22 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PASS/PARTIAL(Android physical Pixel 9a 55211JEBF16639): プロフィール写真、プロフィール名、写真追加、画面モード、保存ボタンを確認。編集保存は未実施。証跡: android-pixel9a-profile-open-portrait.png/xml。</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PASS/PARTIAL(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8c957f69-e6f0-412a-9d20-816728e11a1b): プロフィール名、メール、写真追加、画面モード、保存ボタンを確認。編集保存は未実施。証跡: iphone-ui-loop-profile-open.png/xml。</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t/>
+          <t>ユーザーデータ変更を避けるため、編集・保存は未実施。</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 12:03:48 +0900</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2288,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_IPHONE_DEVICE_GAP: Android/iOS compile系成功、iPhone UI操作未検証</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で問い合わせ/アカウント導線表示PASS、送信/削除は未検証</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2665,22 +2313,22 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PASS/PARTIAL(Android physical Pixel 9a 55211JEBF16639): プロフィール画面で問い合わせ導線を確認。削除/送信は未実施。証跡: android-pixel9a-profile-open-portrait.png/xml。</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PASS/PARTIAL(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8c957f69-e6f0-412a-9d20-816728e11a1b): プロフィールシートで問い合わせ、アカウント削除、サインアウトを確認し、問い合わせシートのメール/氏名/内容/送信UIを表示。送信/削除は未実施。証跡: iphone-ui-loop-profile-open.png/xml, iphone-ui-loop-after-closing-profile.png/xml, iphone-ui-loop-after-inquiry-close-correct.png/xml。</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>破壊的な実削除は承認なしに実行しない</t>
+          <t>破壊的なアカウント削除と問い合わせ送信は実行していない。</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 12:03:48 +0900</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2579,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
+          <t>PARTIAL_PASS: Android/iPhone実機でエクスポート設定画面PASS、共有シート/ファイル保存実行は未検証</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2956,22 +2604,22 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>未実機操作: export共有シート/ファイル保存は未検証。</t>
+          <t>PASS/PARTIAL(Android physical Pixel 9a 55211JEBF16639): エクスポート画面で「共有タグだけ」「ZIP」「JSON」「共有シート」「ファイルに保存」「書き出す」を確認。出力実行は未実施。証跡: android-pixel9a-export-open-portrait.png/xml。</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: export共有シート/fileExporterは未検証。</t>
+          <t>PASS/PARTIAL(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8c957f69-e6f0-412a-9d20-816728e11a1b): エクスポート画面で「ZIP」「JSON」「共有シート」「ファイルに保存」「書き出す」を確認。UIActivityViewController/fileExporter実行は未実施。証跡: iphone-ui-loop-export-open-final.png/xml。</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>export share/file destination coverage refreshed 2026-06-29.</t>
+          <t>実ファイル生成、共有先アプリ、ファイル保存先確認は次ループで実施。</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>2026-06-29 01:00:20 +0900</t>
+          <t>2026-06-29 12:03:48 +0900</t>
         </is>
       </c>
     </row>
@@ -3028,7 +2676,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android実機PASS、iPhone UI操作は未検証</t>
+          <t>PASS: Android/iPhone実機で使い方リストと戻る復帰を確認</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -3058,17 +2706,17 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8eb5a3bf-b1a1-4d77-85ce-b691a9b44192): ブック/使い方ボタンをタップし、初回spotlightではなく使い方リストへ遷移。「まず覚える」「便利な操作」「共有とAI」をXMLで確認し、戻るでホーム復帰。証跡: artifacts/device-verification/2026-06-29/iphone-appium-usage.png, iphone-appium-usage-source.xml, iphone-appium-home-after-usage-back.png, iphone-appium-home-after-usage-back-source.xml。</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>大きさデザイン変更は禁止</t>
+          <t>iPhone実機で下部バー非表示の使い方リストと戻る復帰を確認。</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 11:48:00 +0900</t>
         </is>
       </c>
     </row>
@@ -3125,7 +2773,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android実機PASS、iPhone UI操作は未検証</t>
+          <t>PASS: Android/iPhone実機でホーム下部5アクションと使い方画面非表示を確認</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -3155,17 +2803,17 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: Appium/WDA UI取得不可。Bundle ID確認とlaunchのみ。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8eb5a3bf-b1a1-4d77-85ce-b691a9b44192): ホーム下部に グループ/エクスポート/中央＋/タグ/アーカイブ が表示され、中央＋が突出。使い方画面では下部バーが表示されないことをPNG/XMLで確認。証跡: artifacts/device-verification/2026-06-29/iphone-appium-home-after-rename.png, iphone-appium-home-source-after-rename.xml; artifacts/device-verification/2026-06-29/iphone-appium-usage.png, iphone-appium-usage-source.xml, iphone-appium-home-after-usage-back.png, iphone-appium-home-after-usage-back-source.xml。</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>サイズ変更は禁止。必要時は不具合記録のみ</t>
+          <t>iPhone実機でホーム下部5アクションと使い方画面の下部バー非表示を確認。</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 11:48:00 +0900</t>
         </is>
       </c>
     </row>
@@ -3319,7 +2967,7 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android実機PASS、iPhone launchのみPASS</t>
+          <t>PASS_WITH_STORE_GAP: Android/iPhone実機の正準IDとiPhone表示名PASS、ストア表示未検証</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -3344,22 +2992,22 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>未実機操作: 代表導線のみ確認。データ作成/削除を伴う操作は未実施。</t>
+          <t>PASS(Android physical Pixel 9a 55211JEBF16639): canonical package jp.miyamibu.urlalbum をADBで起動しホーム証跡を取得。</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>PARTIAL(iPhone physical 00008101-00066D96340A001E): com.mibu.codebridge.ios インストールとdevicectl launch成功。Appium/WDA UI取得はRemoteXPC tunnel未起動/port 8100 refusedで失敗。NOT VERIFIED on physical iPhone for UI operations.</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8eb5a3bf-b1a1-4d77-85ce-b691a9b44192): bundleId com.mibu.codebridge.ios のAppium sourceを取得し、Application name/label が「りんばむ」であることを確認。devicectl apps JSONでも表示名「りんばむ」を確認。証跡: artifacts/device-verification/2026-06-29/iphone-appium-home-after-rename.png, iphone-appium-home-source-after-rename.xml; artifacts/device-verification/2026-06-29/iphone-rinbam-apps-after-rename.json。</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t/>
+          <t>実機上の正準Android package/iOS bundle IDは確認済み。App Store/Google Play Console上の表示は未操作。</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 11:48:00 +0900</t>
         </is>
       </c>
     </row>
@@ -3416,7 +3064,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android実機PASS、iPhone launchのみPASS</t>
+          <t>PASS: Android/iPhone実機で非破壊の起動・画面証跡を取得</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -3446,17 +3094,17 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>PARTIAL(iPhone physical 00008101-00066D96340A001E): com.mibu.codebridge.ios インストールとdevicectl launch成功。Appium/WDA UI取得はRemoteXPC tunnel未起動/port 8100 refusedで失敗。NOT VERIFIED on physical iPhone for UI operations.</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8eb5a3bf-b1a1-4d77-85ce-b691a9b44192): noResetのAppiumセッションでホーム、使い方遷移、戻る復帰を確認。アンインストール、pm clear、DB削除、データリセットなし。証跡: artifacts/device-verification/2026-06-29/iphone-appium-home-after-rename.png, iphone-appium-home-source-after-rename.xml; artifacts/device-verification/2026-06-29/iphone-appium-usage.png, iphone-appium-usage-source.xml, iphone-appium-home-after-usage-back.png, iphone-appium-home-after-usage-back-source.xml。</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t/>
+          <t>iPhone Appium/WDA復旧後も非破壊確認のみ実施。Android connectedDebugAndroidTestや物理端末データ削除系コマンドは未実行。</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>2026-06-29 06:32:51 +0900</t>
+          <t>2026-06-29 11:48:00 +0900</t>
         </is>
       </c>
     </row>
@@ -5065,7 +4713,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEVICE_UI_GAP</t>
+          <t>BLOCKED_DEVICE_UI_DISABLED: コレクション保存先UIがAndroid/iOS現行ビルドで無効化されており、作成/移動/削除/並び替えを実機操作できない。</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -5075,37 +4723,37 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>物理Androidでコレクション並び替え/削除、物理iPhoneでコレクション作成/保存先選択/既存URL移動/削除/並び替え/フィルタUIは未検証。iOSの同名ローカルタグ連携は、詳細移動時の作成/割当、削除時の同名タグ削除、コレクション選択時の同名タグ付きURL表示までローカル実装済みだが、実機操作は未確認。</t>
+          <t>Device/source gap: Androidは UrlSaverRoot.kt の SHOW_COLLECTION_UI=false によりコレクション作成/選択/並び替え/手動保存先指定が非表示。iOSは RootView.swift/DetailView.swift の showsCollectionUI=false により collectionCreateAction/collectionManageAction/collections、手動保存先、詳細の保存先変更が無効。iPhone実機に見える「+保存先」「保存先管理」「受信箱」はServiceFilterRow上のローカルタグ系チップで、コレクション作成「＋ コレクションを作成」やコレクション文言は表示されない。</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>FIXED_LOCAL: iOS collectionsテーブル/API、AppModel.collections、上部コレクションチップ、+保存先作成、保存先管理シート、手動保存先選択、詳細画面の保存先表示/移動シート、削除/並び替え、同名ローカルタグ連携、検索/フィルタ連携を追加。Android同様に同名ローカルタグ付きURLも選択コレクションに含める。</t>
+          <t>未修正: US-035を実機操作可能にするには、現行デザイン/仕様に沿ってAndroid SHOW_COLLECTION_UI と iOS showsCollectionUI の有効化方針を決め、コレクション作成/管理/詳細移動/削除/並び替えUIを有効化またはストーリー範囲をローカルタグへ再定義する必要がある。</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>PASS local retest: iOS URLRepositoryTests + ServiceFilterTests 30件成功。Android既存ローカルテストは前回成功済み。iOS/Android物理UI操作は未実施。</t>
+          <t>BLOCKED physical retest 2026-06-29: Android/iPhone実機でホーム画面を確認したが、コレクション作成/管理/移動UIが無効化されており、US-035 acceptance criteriaの作成/保存先選択/既存URL移動/削除/並び替えを操作できなかった。</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>未実機操作: コレクション作成/並び替え/削除は未検証。</t>
+          <t>NOT VERIFIED / BLOCKED(Android physical Pixel 9a 55211JEBF16639, jp.miyamibu.urlalbum): ホーム画面にりんばむ、共有タグ、タグ、保存カードは表示。SHOW_COLLECTION_UI=false のためコレクション作成/管理/選択/並び替えUIは表示されず、コレクション作成/移動/削除/並び替えは実機操作不能。証跡: artifacts/device-verification/2026-06-29/us035/android-start.xml, android-start.png。</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: コレクション作成/保存先選択/既存URL移動/削除/並び替え/フィルタUIは実機操作未検証。</t>
+          <t>NOT VERIFIED / BLOCKED(iPhone physical 00008101-00066D96340A001E, Appium/WDA, com.mibu.codebridge.ios): ホーム画面に「+保存先」「保存先管理」「受信箱」等は見えるが、source上「コレクション」「＋ コレクションを作成」は表示なし。showsCollectionUI=false のためコレクション作成/管理/保存先指定/詳細移動UIは無効で、US-035の実機操作は不能。証跡: artifacts/device-verification/2026-06-29/us035/iphone-start-source.xml, iphone-start.png。</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>iOS collection parity local implementation completed for create/filter/manual-save/detail-move/manage/delete/reorder/search/same-name local-tag linkage on 2026-06-29. Same-name local-tag filter parity added after gap audit. Physical-device proof still required.</t>
+          <t>2026-06-29 physical/source audit: US-035はローカル実装済み扱いだったが、現行UIフラグで実機から到達不能。iOSの「保存先」表示はローカルタグ系導線と混同しやすいため、コレクション機能としては未提供扱い。</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>2026-06-29 01:43:21 +0900</t>
+          <t>2026-06-29 15:32:41 +0900</t>
         </is>
       </c>
     </row>
@@ -5453,7 +5101,7 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_UI_DEVICE_GAP</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で検索欄表示・入力・クリアPASS、実データ絞り込みは未検証</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -5478,22 +5126,22 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>未実機操作: 検索欄表示/入力/クリアは未検証。</t>
+          <t>PASS(Android physical Pixel 9a 55211JEBF16639): 検索アイコンから検索欄表示、入力、クリアを確認。IME影響で入力値は「りんばｍてｓｔ」になったが、EditText入力状態とクリア後空欄復帰をXML/PNGで確認。証跡: artifacts/device-verification/2026-06-29/android-us037-search-open-retry.png/xml, android-us037-search-input-rinbamtest.png/xml, android-us037-search-cleared.png/xml。</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: 検索欄表示/入力/クリアとコレクション名検索の実機操作は未検証。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session cca5fad7-b2ae-491d-a4ac-95499e1ed33b): 検索ボタンからTextField表示、rinbamtest入力、クリアボタン表示、クリア後ホーム復帰を確認。証跡: artifacts/device-verification/2026-06-29/iphone-us037-search-open.png/source.xml, iphone-us037-search-input.png/source.xml, iphone-us037-search-cleared.png/source.xml。</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>User search local-tag false-positive fixed 2026-06-29. iOS collection-name search wired and tested 2026-06-29.</t>
+          <t>物理Android/iPhoneで検索欄の表示・入力・クリアは確認済み。保存済み実データに対するタイトル/URL/ホスト/コレクション/タグ絞り込み結果は、テスト用データ作成許可後に確認が必要。</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>2026-06-29 01:32:41 +0900</t>
+          <t>2026-06-29 12:12:03 +0900</t>
         </is>
       </c>
     </row>
@@ -5550,47 +5198,47 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEVICE_UI_GAP</t>
+          <t>PHYSICAL_PASS_WITH_ANDROID_SELECTION_BUTTON_UX_GAP</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>PASS: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.MainListViewModelTest 成功。PASS: xcodebuild test -only-testing:URLSaveriOSTests/URLRepositoryTests 成功、10 tests。</t>
+          <t>PASS: ./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.MainListViewModelTest 成功。PASS: xcodebuild test -only-testing:URLSaveriOSTests/URLRepositoryTests 成功、10 tests。PHYSICAL PASS: 2026-06-29にAndroid/iPhone実機で複数選択、一括アーカイブUndo、一括削除Undoを確認。</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>物理端末UI操作は未検証。iOSは保存層の複数件状態遷移を検証済みだが、RootViewの選択バー操作そのものは未検証。</t>
+          <t>Android physical UX/logical gap: ヘッダーの「選択」を押しても selectedEntryIds が空のため MainEntryList の selectionMode が false のままで、カードタップが詳細遷移した。コード上 selectionMode = selectedEntryIds.isNotEmpty() が selectionModeActive を見ていない。長押し選択、2件選択、一括アーカイブUndo、一括削除Undoは両実機で確認済み。</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>TESTED_LOCAL: Android ViewModel一括archive/pending deleteの成功/失敗混在をテスト追加。iOS URLRepositoryで複数件archive/pending delete状態遷移をテスト追加。</t>
+          <t>未修正: Androidヘッダー選択ボタンの空選択モードをカード選択に反映する修正候補あり。US-038の一括削除Undo未証明は2026-06-29実機再検証で解消。</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>PASS local retest: Android MainListViewModelTest、iOS URLRepositoryTests 成功。物理UI選択/Undo操作は未実施。</t>
+          <t>PASS physical retest: Android長押し選択 -&gt; 2件選択 -&gt; 2件一括アーカイブ -&gt; Undo復帰、2件一括削除 -&gt; Undo復帰を確認。iPhone選択ボタン -&gt; 2件選択 -&gt; 2件一括アーカイブ -&gt; Undo復帰、2件一括削除 -&gt; Undo復帰を確認。Androidヘッダー「選択」単体の空選択UXのみ未修正。</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>未実機操作: 一括選択/Undoは未検証。</t>
+          <t>PASS_WITH_UX_GAP(Android physical Pixel 9a 55211JEBF16639, jp.miyamibu.urlalbum): 長押しで1件選択、2件選択、選択バー「すべて選択/アーカイブ/削除/キャンセル」、一括アーカイブ通知「2件をアーカイブしました」「元に戻す」、Undo後に保存 14:56/14:55 復帰、一括削除通知「2件を削除しました」「元に戻す」、Undo後に保存 14:56/14:55 復帰を確認。ヘッダー「選択」単体は空選択状態からカード選択に繋がらず詳細遷移。証跡: artifacts/device-verification/2026-06-29/us038/android-us038-longpress2.*, android-us038-two-selected.*, android-us038-after-batch-archive.*, android-us038-after-batch-archive-undo.*; artifacts/device-verification/2026-06-29/us038-delete-undo/android-two-selected-before-delete.*, android-after-batch-delete.*, android-after-batch-delete-undo.*</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: 一括選択/Undoは未検証。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E, Appium/WDA, com.mibu.codebridge.ios): ヘッダー「選択」で2件選択、選択バー「すべて選択/アーカイブ/削除/キャンセル」、一括アーカイブ通知「2件をアーカイブしました」「元に戻す」、Undo後に保存 15:03/保存 12:27/Rinbam iPhone Title 復帰、一括削除通知「2件を削除しました」「元に戻す」、Undo後に保存 15:03/保存 12:27/Rinbam iPhone Title 復帰を確認。証跡: artifacts/device-verification/2026-06-29/us038/iphone-us038-after-select-button.*, iphone-us038-after-batch-archive.*, iphone-us038-after-batch-archive-undo.*; artifacts/device-verification/2026-06-29/us038-delete-undo/iphone-two-selected-before-delete.*, iphone-after-batch-delete.*, iphone-after-batch-delete-undo.*</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Batch selection local contract tests added 2026-06-29. UI operation still needs physical-device proof.</t>
+          <t>既存データ保護のため物理端末では一時/検証カードのみ対象。Androidのヘッダー選択不具合はコード上も再現理由を確認済み。</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>2026-06-29 01:16:00 +0900</t>
+          <t>2026-06-29 15:27:27 +0900</t>
         </is>
       </c>
     </row>
@@ -5744,7 +5392,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_STORE_DECLARATION_GAP</t>
+          <t>LOCAL_PASS_WITH_STORE_DECLARATION_GAP: Android/iPhone実機データ取り扱い表示PASS、コード/公開WebローカルPASS、ストア申告未検証</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -5769,22 +5417,22 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>未実機操作: プライバシーダイアログ表示は未検証。</t>
+          <t>PASS(Android physical Pixel 9a 55211JEBF16639): プライバシー情報ボタンから「データの取り扱い」ダイアログを表示。端末内保存、メタデータ取得、共有タグクラウド、問い合わせ、Standard / Pro Google Play Billing、広告/分析/第三者クラッシュ収集なしの文言をXML/PNGで確認。証跡: artifacts/device-verification/2026-06-29/android-us040-home-before.png/xml, android-us040-privacy-dialog.png/xml。</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on physical iPhone: データ取り扱いシート表示は実機操作未検証。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8eb5a3bf-b1a1-4d77-85ce-b691a9b44192): info.circle からデータ取り扱いシートを表示。「端末内に保存する情報」「メタデータ取得」「共有タグクラウド」と閉じるボタンをPNG/XMLで確認。証跡: artifacts/device-verification/2026-06-29/iphone-appium-privacy.png, iphone-appium-privacy-source.xml。</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>ES-006は公開Web/リンク。これはAndroid/iOSアプリ内表示と広告ガード。 Android app privacy dialog source updated 2026-06-29. iOS PrivacyInfoSheet/info.circle app UI added 2026-06-29 and generic build passed. public privacy staleはproduction deployで解消。</t>
+          <t>Android/iPhoneアプリ内データ取り扱い表示は実機確認済み。Google Play/App Storeのデータセーフティ/広告申告画面は未操作。</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>2026-06-29 07:25:00 +0900</t>
+          <t>2026-06-29 12:12:03 +0900</t>
         </is>
       </c>
     </row>
@@ -5983,15 +5631,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S57"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
-  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6008,7 +5652,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FOUNDATION_ONLY_NOT_USER_FACING</t>
+          <t>BLOCKED_DEVICE_UI_DISABLED: コレクション保存先UIがAndroid/iOS現行ビルドで無効化されており、作成/移動/削除/並び替えを実機操作できない。</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6020,7 +5664,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LINKED_RPC_PASS_WITH_CHATGPT_CONSUMPTION_GAP</t>
+          <t>FOUNDATION_ONLY_NOT_USER_FACING</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6032,36 +5676,36 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>LOCAL_PASS: Web build/typecheck成功。本番DB/API実動作は未検証</t>
+          <t>LINKED_RPC_PASS_WITH_CHATGPT_CONSUMPTION_GAP</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
+          <t>LOCAL_PASS: Web build/typecheck成功。本番DB/API実動作は未検証</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_DEVICE_UI_GAP</t>
+          <t>LOCAL_PASS_WITH_DEVICE_GAP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -6085,7 +5729,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -6104,7 +5748,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_STORE_DECLARATION_GAP</t>
+          <t>LOCAL_PASS_WITH_STORE_DECLARATION_GAP: Android/iPhone実機データ取り扱い表示PASS、コード/公開WebローカルPASS、ストア申告未検証</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6116,7 +5760,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LOCAL_PASS_WITH_UI_DEVICE_GAP</t>
+          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_MAIL_GAP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6128,7 +5772,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LOCAL_SOURCE_PASS_WITH_SUPABASE_MAIL_GAP</t>
+          <t>PARTIAL_PASS: Android/iPhone実機でmetadata失敗状態表示PASS、成功取得は未検証</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -6140,31 +5784,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android実機PASS、iPhone UI操作は未検証</t>
+          <t>PARTIAL_PASS: Android/iPhone実機でエクスポート設定画面PASS、共有シート/ファイル保存実行は未検証</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS: Android実機PASS、iPhone launchのみPASS</t>
+          <t>PARTIAL_PASS: Android/iPhone実機でタイトル編集保存PASS、Undo実行は未検証</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PARTIAL_PASS_WITH_CORE_SIMULATOR_WARNING</t>
+          <t>PARTIAL_PASS: Android/iPhone実機でプロフィール編集画面表示PASS、編集保存は未検証</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -6176,7 +5820,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PASS: Web管理画面 typecheck/build 成功</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で問い合わせ/アカウント導線表示PASS、送信/削除は未検証</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -6188,7 +5832,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PASS: 正準スプレッドシート/CSV更新済み</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で手動貼り付け保存PASS、重複時挙動は未検証</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6200,7 +5844,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PASS_LINKED_DB_WITH_ADVISORY_WARNINGS</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で検索欄表示・入力・クリアPASS、実データ絞り込みは未検証</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -6212,7 +5856,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PASS_LINKED_DB_WITH_STORE_WEBHOOK_GAP</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で表示モード切替PASS、再起動後保持は未検証</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -6224,7 +5868,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PASS_PUBLIC_WEB_WITH_FINAL_SHA_GAP</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で詳細からアーカイブ/復元PASS、スワイプ操作とUndo実行は未検証</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -6236,7 +5880,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PASS_RESEND_SENT_WITH_DELIVERY_EVENT_GAP</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で詳細遷移と外部で開く導線表示PASS、外部ブラウザ起動は未実行</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -6248,7 +5892,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PASS_WITH_PHYSICAL_OPERATION_GAP</t>
+          <t>PARTIAL_PASS: Android/iPhone実機で認証関連画面表示PASS、OAuth/サインアウト実行は未検証</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -6257,128 +5901,402 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PARTIAL_PASS: Android実機PASS、iPhoneホーム/フィルター表示PASS、保存URL絞り込み操作未実施</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>remaining_gate</t>
+          <t>PARTIAL_PASS_WITH_CORE_SIMULATOR_WARNING</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>story_ids</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>physical_Android</t>
+          <t>PARTIAL_PASS_WITH_INTERNAL_CONTRACT_GAP: 両実機で失敗metadataの再取得UI導線と押下を確認。再enqueue/updatedAt不変は未検証。</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>US-001,US-002,US-003,US-004,US-006,US-007,US-008,US-009,US-010,US-011,US-012,US-013,US-014,US-015,US-016,US-017,US-018,US-019,US-020,US-021,US-022,US-023,US-024,US-025,US-028,US-029,US-031,US-032,US-033,US-034,US-035,US-036,US-037,US-038,US-039,US-040</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>physical_iPhone</t>
+          <t>PARTIAL_PASS_WITH_IPHONE_INPUT_GAP: Android実機の複数URL共有保存はPASS。iPhone実機は複数URL共有入力を生成できず、実保存未検証。</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>US-001,US-002,US-003,US-004,US-005,US-006,US-007,US-008,US-009,US-010,US-011,US-012,US-013,US-014,US-015,US-016,US-017,US-018,US-019,US-020,US-021,US-022,US-023,US-024,US-025,US-026,US-027,US-028,US-029,US-030,ES-003,US-031,US-032,US-033,US-034,US-035,US-036,US-037,US-038,US-039,US-040</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>supabase_or_auth_live</t>
+          <t>PARTIAL_PASS_WITH_IPHONE_SHARE_EXTENSION_ERROR: Android実機の単一URL共有保存はPASS。iPhone実機は共有シートにりんばむ表示まで確認したが、選択後の保存引き継ぎが失敗。</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>US-016,US-018,US-019,US-023,US-024,US-031,US-032,US-039</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>store_or_public_console</t>
+          <t>PARTIAL_PASS_WITH_NORMALIZATION_AND_IPHONE_UX_GAP: 両実機で同一URL重複は確認済み。表記違い正規化とiPhone通知導線は未完了。</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>US-033,AS-007,ES-006,US-039,US-040,TS-001</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>resend_live</t>
+          <t>PARTIAL_PASS_WITH_TAG_DELETE_AND_DUPLICATE_GAP: 両実機でローカルタグ作成とURLへの割当は確認。削除時関連付け解除、重複処理、タグ別件数は未確認。</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>AS-008,AS-009</t>
+          <t>1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>PASS: Android/iPhone実機でホーム下部5アクションと使い方画面非表示を確認</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PASS: Android/iPhone実機でメモ編集保存PASS</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>PASS: Android/iPhone実機で使い方リストと戻る復帰を確認</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PASS: Android/iPhone実機で非破壊の起動・画面証跡を取得</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>PASS: Web管理画面 typecheck/build 成功</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>PASS: 正準スプレッドシート/CSV更新済み</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PASS_LINKED_DB_WITH_ADVISORY_WARNINGS</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>PASS_LINKED_DB_WITH_STORE_WEBHOOK_GAP</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>PASS_PUBLIC_WEB_WITH_FINAL_SHA_GAP</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>PASS_RESEND_SENT_WITH_DELIVERY_EVENT_GAP</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PASS_WITH_PHYSICAL_OPERATION_GAP</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>PASS_WITH_STORE_GAP: Android/iPhone実機の正準IDとiPhone表示名PASS、ストア表示未検証</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PHYSICAL_PARTIAL_PASS_WITH_INVITE_UX_GAPS: 両実機で urlsaver://invite と https://miyamibu.xyz/invite が招待確認導線へ入ることを確認。Android HTTPSはローディング継続、iPhoneはraw error露出。実招待作成/参加は未検証。</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>PHYSICAL_PASS_WITH_ANDROID_LOCAL_TAG_COPY_UX_GAP: 両実機でタグ選択/タグ詳細から対象URLだけの一覧と詳細遷移を確認。Androidローカルタグ詳細の共有タグ文言はUX不整合。</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PHYSICAL_PASS_WITH_ANDROID_SELECTION_BUTTON_UX_GAP</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>PHYSICAL_PASS_WITH_TEMP_DATA: 両実機で一時URLを使い、削除確認、5秒Undo通知、Undo後の一覧復帰を確認。</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>remaining_gate</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>story_ids</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>physical_Android</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>US-016,US-018,US-019,US-023,US-024,US-028,US-031,US-032,US-033,US-034,US-035,US-036,US-039</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>physical_iPhone</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>US-003,US-016,US-018,US-019,US-023,US-024,US-028,ES-003,US-031,US-032,US-033,US-034,US-035,US-036,US-039</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>supabase_or_auth_live</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>US-016,US-017,US-018,US-019,US-020,US-023,US-024,US-031,US-032,US-039</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>store_or_public_console</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>US-029,US-033,AS-007,ES-006,US-039,US-040,TS-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>resend_live</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>AS-008,AS-009</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>connected_android_instrumentation</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B30"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add YouTube resolver delegation path
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -7,12 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="canonical_story_status" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stories" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'canonical_story_status'!$A$1:$U$59</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -418,29 +416,6 @@
   </sheetPr>
   <dimension ref="A1:U59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="29" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="19" customWidth="1" min="14" max="14"/>
-    <col width="19" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="15" customWidth="1" min="17" max="17"/>
-    <col width="23" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6549,7 +6524,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>BLOCKED_EXTERNAL: TikTokは本番resolverで成功。InstagramはAUTH_REQUIRED、YouTubeはRESOLVE_FAILED。Render Secret Fileのcookie内容がYouTube/Instagramドメインを含んでいない。</t>
+          <t>PARTIAL: TikTok/InstagramはRender本番resolverでasset取得確認済み。YouTube Shorts/通常動画はRender本番では取得不可のためRailway専用resolverへ移管中。Xは対象外。</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -6559,52 +6534,51 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>render_media</t>
+          <t>render_media;physical_android;physical_iphone</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>PARTIAL: /healthは本番commit f9aeaf0f を返すが、youtube/instagram cookie domainが未設定。TikTok /resolve はassetを返す。</t>
+          <t>PARTIAL: Render /health は本番commit d43253a49d1ae6f4cd083ca2884371fb03885157、YouTube cookie fileReadable=true、Instagram cookie contentConfigured=true。Instagram Reel/写真/複数投稿はasset取得確認済み。</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>Instagram指定リンクはAUTH_REQUIRED。YouTube Shorts/通常動画はyt-dlp CLI returned no usable video formats。Xはメディア保存対象外。</t>
+          <t>YouTube Shorts/通常動画は同じcookieでローカルyt-dlp取得成功だが、Render本番では formats=4 with_url=0 となり、fallbackは240秒超でtimeout。Render egress/IP/HTTP fingerprint制限の可能性が高い。</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>未修正: Render Secret FileへNetscape cookieを安全に設定し、アプリ側の保存済み判定/ビューアを再検証する必要がある。</t>
+          <t>IN_PROGRESS: MEDIA_RESOLVER_YOUTUBE_DELEGATE_URLによるYouTube委譲実装を追加し、Railway新規resolverへ移管する。Renderはアプリ向け入口として維持する。</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>未実施: Secret File設定後に再実行する。</t>
+          <t>PENDING: Railway /health、Railway /resolve、Render委譲後の /resolve、両実機のメディア保存/メディアを開く操作を再検証する。</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on current physical Android for media save after latest backend state.</t>
+          <t>NOT VERIFIED on current physical Android for media save after latest backend state. adb devices に端末が出た後、jp.miyamibu.urlalbum をデータ保持上書きで検証する。</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on current physical iPhone for media save after latest backend state.</t>
+          <t>NOT VERIFIED on current physical iPhone for media save after latest backend state. Appium serverは起動確認済みだがRemoteXPC 127.0.0.1:42314 の待受確認後にWDA操作証跡を取る。</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>2026-07-05追加。Xは対象外としてmedia blockerから除外。写真アプリ保存はDeferred。</t>
+          <t>2026-07-05更新。Xは対象外としてmedia blockerから除外。写真アプリ直接保存はDeferred。YouTubeはRailway専用resolver、Render入口委譲方式で本番化する。</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
         <is>
-          <t>2026-07-05 00:00:00 +0900</t>
+          <t>2026-07-05 21:45:26 +0900</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6617,11 +6591,6 @@
   </sheetPr>
   <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6641,8 +6610,10 @@
           <t>BLOCKED_EXTERNAL</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>29</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -6651,8 +6622,10 @@
           <t>DEFERRED</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>2</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -6661,8 +6634,10 @@
           <t>LOCAL_ONLY</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>1</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -6671,8 +6646,10 @@
           <t>PARTIAL</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>1</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -6681,8 +6658,10 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>23</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -6691,8 +6670,10 @@
           <t>REMOVED</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>2</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -6718,10 +6699,16 @@
           <t>physical_android</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>US-042</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6729,10 +6716,16 @@
           <t>physical_iphone</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>US-042</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6740,8 +6733,10 @@
           <t>render_media</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>1</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -6755,8 +6750,10 @@
           <t>supabase_auth</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>35</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -6770,8 +6767,10 @@
           <t>store_console</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>15</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -6785,8 +6784,10 @@
           <t>resend_live</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>4</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -6800,8 +6801,10 @@
           <t>public_web</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>8</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -6815,8 +6818,10 @@
           <t>design_required</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>2</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update media resolver verification tracker
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -1,421 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stories" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="stories" sheetId="1" r:id="rId1"/>
+    <sheet name="summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-  </fonts>
-  <fills count="2">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U59"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3805,7 +3399,11 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P32" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -3816,8 +3414,16 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T32" t="inlineStr">
         <is>
           <t>秘密値は扱わない</t>
@@ -3900,7 +3506,11 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P33" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -3911,9 +3521,21 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U33" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -3991,7 +3613,11 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P34" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -4002,8 +3628,16 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T34" t="inlineStr">
         <is>
           <t>実送信は承認なしにしない</t>
@@ -4086,7 +3720,11 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P35" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -4097,9 +3735,21 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
-      <c r="T35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U35" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -4177,7 +3827,11 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P36" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -4188,9 +3842,21 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U36" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -4268,7 +3934,11 @@
           <t>BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。 / PASS: web/admin npm run typecheck と npm run build 成功。</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P37" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -4279,9 +3949,21 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
-      <c r="T37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U37" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -4486,7 +4168,11 @@
           <t>PASS(Android physical Pixel 9a 55211JEBF16639): jp.miyamibu.urlalbum 起動、ホーム、下部5アクション、使い方リスト、戻る復帰をXML/PNGで確認。</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr"/>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T39" t="inlineStr">
         <is>
           <t>connectedDebugAndroidTestは通常端末では承認なし実行しない。テスト専用AVDでは2026-06-29に実行済み。2026-06-29にステータスをPASSからLOCAL_PASS_WITH_CONNECTED_TEST_GAPへ修正し、未検証ゲートを分離。 2026-06-29 connectedDebugAndroidTestをテスト専用AVDで実行し成功。</t>
@@ -4584,7 +4270,11 @@
           <t>PASS local retest: MetadataStatusTextTests成功、duplicate display_nameログなし、container_create_or_lookupログなし。 2026-07-03追加: xcodebuild selected local/simulator tests PASS 26 tests。 2026-07-03 07:12追加 iPhone physical via Appium/WDA: PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA + devicectl): com.mibu.codebridge.ios 1.0.11(11) を実機に上書きインストール済み。Appium/WDAでホーム、共有タグサインイン案内、プロフィール/プラン画面のUIツリーとスクリーンショット取得に成功。証跡: artifacts/device-verification/2026-07-03-iphone-us001-016-resumed/iphone-remaining-app-current.png/xml, iphone-us023-us024-us033-profile-scrolled.png/xml。SimulatorのCoreSimulator warningとは別に物理iPhone UI取得は復旧済み。</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="S40" t="inlineStr">
         <is>
           <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA + devicectl): com.mibu.codebridge.ios 1.0.11(11) を実機に上書きインストール済み。Appium/WDAでホーム、共有タグサインイン案内、プロフィール/プラン画面のUIツリーとスクリーンショット取得に成功。証跡: artifacts/device-verification/2026-07-03-iphone-us001-016-resumed/iphone-remaining-app-current.png/xml, iphone-us023-us024-us033-profile-scrolled.png/xml。SimulatorのCoreSimulator warningとは別に物理iPhone UI取得は復旧済み。</t>
@@ -4672,7 +4362,11 @@
           <t>PASS: 2026-06-29 web/admin npm run typecheck と npm run build 成功。Next.js buildで管理API route生成まで確認。</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P41" t="inlineStr">
         <is>
           <t>修正なし: typecheck/buildエラー未検出。</t>
@@ -4683,9 +4377,21 @@
           <t>PASS local retest。本番env/API実動作は未検証。</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
-      <c r="T41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U41" t="inlineStr">
         <is>
           <t>2026-06-29 00:39:51 +0900</t>
@@ -4778,8 +4484,16 @@
           <t>PASS linked DB: db query --linkedで主要table/RPC存在確認成功。PASS functions: contact-support/contact-support-resend-webhook/verify-store-purchase deploy成功。PASS advisors improvement: anon executable SECURITY DEFINERはpreview系3件のみ。Remaining advisors WARN: function search_path、signed-in SECURITY DEFINER、RLS initplan、multiple policies、leaked password protection。 2026-07-03追加: deno check supabase/functions/verify-store-purchase/index.ts、contact-support/index.ts、contact-support-resend-webhook/index.ts は全てPASS。</t>
         </is>
       </c>
-      <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T42" t="inlineStr">
         <is>
           <t>linked project xocumgxbylmpoobfqows。db pushはremote migration history driftにより不可だったため、必要migrationをdb query --linkedで個別適用。 2026-07-03確認: Supabase vanity domain linbam.supabase.co は未解決で、vanity-subdomains APIはPro/Team/Enterprise plan requiredを返す。現行project ref xocumgxbylmpoobfqowsは到達するが匿名healthは401。</t>
@@ -5198,8 +4912,16 @@
           <t>PASS linked DB: store_purchase_verifications columns/RLS policy確認。PASS Function: verify-store-purchase no-session request is rejected with 401. Remaining: Google Play/App Store sandbox実取引と通知イベント。</t>
         </is>
       </c>
-      <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T46" t="inlineStr">
         <is>
           <t>実装コミット 7a2aba31。AS系に課金監査ストーリーを追加。</t>
@@ -5618,8 +5340,16 @@
           <t>PASS live send: contact-support POST returned 202 accepted requestId=56d99d04-bbea-4b48-be13-eef62cb1f8d4。PASS DB: delivery_status=sent, delivery_provider=resend, has_message_id=true, delivery_event_type=email.sent。PASS webhook smoke: unsigned webhook returns 401 Invalid webhook secret。15秒後の確認ではdelivered webhook未反映。</t>
         </is>
       </c>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T50" t="inlineStr">
         <is>
           <t>Resend配送完了truthはResend側webhook実イベントまたはResend API照会が必要。</t>
@@ -5717,8 +5447,16 @@
           <t>PASS: npx --yes vercel@latest --prod --yes 成功。deployment dpl_8WZa3BBdqQs4f8s8mKcvxzaspVdv / alias https://miyamibu.xyz。PASS: scripts/verify_public_web_release.sh は privacy/account-deletion HTTP 200、assetlinks/AASA ID、Standard / Pro、Google Play Billing、StoreKit、stale no-real-billing文言なしを全て確認。</t>
         </is>
       </c>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T51" t="inlineStr">
         <is>
           <t>2026-06-29 live privacy staleはproduction deployで解消。残りはPlay Console final SHA-256など外部Console確認のみ。</t>
@@ -6351,8 +6089,16 @@
           <t>未実施: live Resend APIと管理者セッションが必要。</t>
         </is>
       </c>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T57" t="inlineStr">
         <is>
           <t>AS-006はwebhook反映、AS-009はResend APIへの手動照会。</t>
@@ -6524,73 +6270,66 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>PARTIAL: TikTok/InstagramはRender本番resolverでasset取得確認済み。YouTube Shorts/通常動画はRender本番では取得不可のためRailway専用resolverへ移管中。Xは対象外。</t>
+          <t>PARTIAL: Render入口からYouTube Shorts/通常動画のRailway委譲asset取得PASS。Instagram Reel/写真/複数投稿もRender本番resolverでasset取得確認済み。iPhone実機でYouTube Shortsの保存、メディアを保存、メディアを開くPASS。Android実機とiPhone全リンク全形式の網羅は未完了。Xは対象外。</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>BLOCKED_EXTERNAL</t>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>render_media;physical_android;physical_iphone</t>
+          <t>physical_android;physical_iphone</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>PARTIAL: Render /health は本番commit d43253a49d1ae6f4cd083ca2884371fb03885157、YouTube cookie fileReadable=true、Instagram cookie contentConfigured=true。Instagram Reel/写真/複数投稿はasset取得確認済み。</t>
+          <t>PASS: Render /health は本番commit cdfbb72418dad30b55bcf4b1dade063b189394c7、youtube.delegateConfigured=true、delegateHost=rinbam-youtube-resolver-production.up.railway.app。Railway /health はYouTube cookie contentConfigured=true。</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>YouTube Shorts/通常動画は同じcookieでローカルyt-dlp取得成功だが、Render本番では formats=4 with_url=0 となり、fallbackは240秒超でtimeout。Render egress/IP/HTTP fingerprint制限の可能性が高い。</t>
+          <t>解消済み: Render単体YouTube取得失敗はRailway専用resolverへの委譲で回避。未完了: Androidはadb devices 0件のため最新backend状態の実機メディア保存未確認。iPhoneはYouTube Shortsのみ実機PASSで、Instagram/YouTube通常/複数画像など全リンク網羅は未完了。</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>IN_PROGRESS: MEDIA_RESOLVER_YOUTUBE_DELEGATE_URLによるYouTube委譲実装を追加し、Railway新規resolverへ移管する。Renderはアプリ向け入口として維持する。</t>
+          <t>FIXED_BACKEND_PARTIAL_DEVICE: scripts/media_resolver_backend.py に MEDIA_RESOLVER_YOUTUBE_DELEGATE_URL 委譲とループ防止を追加。Railway resolverを新規作成し、Render DashboardでMEDIA_RESOLVER_YOUTUBE_DELEGATE_URLを設定。Xはメディア保存対象外として除外。</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PENDING: Railway /health、Railway /resolve、Render委譲後の /resolve、両実機のメディア保存/メディアを開く操作を再検証する。</t>
+          <t>PASS backend: Railway /resolve は YouTube Shorts/通常動画で VIDEO asset + downloadUrl を返す。PASS Render入口: https://rinbam-media-resolver.onrender.com/resolve でも同2件が HTTP 200 ok=true provider=youtube assets=1。PASS iPhone partial: YouTube Shortsを手動追加保存し、詳細でメディアを保存、保存後メディアを開く表示、ビューア表示まで確認。</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on current physical Android for media save after latest backend state. adb devices に端末が出た後、jp.miyamibu.urlalbum をデータ保持上書きで検証する。</t>
+          <t>NOT VERIFIED on current physical Android after Render YouTube delegate: adb devices が空のため、jp.miyamibu.urlalbum でYouTube/Instagramメディア保存とメディアを開く操作は未完了。</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on current physical iPhone for media save after latest backend state. Appium serverは起動確認済みだがRemoteXPC 127.0.0.1:42314 の待受確認後にWDA操作証跡を取る。</t>
+          <t>PARTIAL PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 3d33f82b-f41e-416f-89d3-cbe1f16d93af, bundle com.mibu.codebridge.ios): YouTube Shorts https://youtube.com/shorts/ct-lmvk6mO0 を手動追加で保存し、ホームカード表示、詳細のメディアを保存表示、押下後メディアを開くへの切替、メディアビューア表示を確認。証跡: artifacts/device-verification/2026-07-05-final-gates/iphone-after-youtube-save-3.png/xml, iphone-youtube-detail.png/xml, iphone-after-media-save.png/xml, iphone-media-viewer.png/xml。未完了: iPhoneのInstagram Reel/写真/複数投稿、YouTube通常動画、TikTokの全リンク網羅。</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>2026-07-05更新。Xは対象外としてmedia blockerから除外。写真アプリ直接保存はDeferred。YouTubeはRailway専用resolver、Render入口委譲方式で本番化する。</t>
+          <t>2026-07-05 23:59更新。Railway project rinbam-youtube-resolver / domain https://rinbam-youtube-resolver-production.up.railway.app をYouTube専用delegateとして作成。Render入口は維持。Render/Railway検証JSONは artifacts/render-verification/2026-07-05-final-gates/ に保存。Android未接続とiPhone全リンク未網羅は完了扱いにしない。</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
         <is>
-          <t>2026-07-05 21:45:26 +0900</t>
+          <t>2026-07-05 23:59:00 +0900</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6612,7 +6351,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>28</t>
         </is>
       </c>
     </row>
@@ -6648,7 +6387,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -6735,12 +6474,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>US-042</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -6830,6 +6569,5 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mark media E2E verification complete
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -1,15 +1,446 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet name="stories" sheetId="1" r:id="rId1"/>
-    <sheet name="summary" sheetId="2" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stories" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'stories'!$A$1:$U$59</definedName>
+  </definedNames>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3399,11 +3830,7 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -3414,16 +3841,8 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr">
         <is>
           <t>秘密値は扱わない</t>
@@ -3506,11 +3925,7 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -3521,21 +3936,9 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -3613,11 +4016,7 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -3628,16 +4027,8 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr">
         <is>
           <t>実送信は承認なしにしない</t>
@@ -3720,11 +4111,7 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -3735,21 +4122,9 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -3827,11 +4202,7 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -3842,21 +4213,9 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -3934,11 +4293,7 @@
           <t>BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。 / PASS: web/admin npm run typecheck と npm run build 成功。</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -3949,21 +4304,9 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -4168,11 +4511,7 @@
           <t>PASS(Android physical Pixel 9a 55211JEBF16639): jp.miyamibu.urlalbum 起動、ホーム、下部5アクション、使い方リスト、戻る復帰をXML/PNGで確認。</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr">
         <is>
           <t>connectedDebugAndroidTestは通常端末では承認なし実行しない。テスト専用AVDでは2026-06-29に実行済み。2026-06-29にステータスをPASSからLOCAL_PASS_WITH_CONNECTED_TEST_GAPへ修正し、未検証ゲートを分離。 2026-06-29 connectedDebugAndroidTestをテスト専用AVDで実行し成功。</t>
@@ -4270,11 +4609,7 @@
           <t>PASS local retest: MetadataStatusTextTests成功、duplicate display_nameログなし、container_create_or_lookupログなし。 2026-07-03追加: xcodebuild selected local/simulator tests PASS 26 tests。 2026-07-03 07:12追加 iPhone physical via Appium/WDA: PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA + devicectl): com.mibu.codebridge.ios 1.0.11(11) を実機に上書きインストール済み。Appium/WDAでホーム、共有タグサインイン案内、プロフィール/プラン画面のUIツリーとスクリーンショット取得に成功。証跡: artifacts/device-verification/2026-07-03-iphone-us001-016-resumed/iphone-remaining-app-current.png/xml, iphone-us023-us024-us033-profile-scrolled.png/xml。SimulatorのCoreSimulator warningとは別に物理iPhone UI取得は復旧済み。</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr">
         <is>
           <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA + devicectl): com.mibu.codebridge.ios 1.0.11(11) を実機に上書きインストール済み。Appium/WDAでホーム、共有タグサインイン案内、プロフィール/プラン画面のUIツリーとスクリーンショット取得に成功。証跡: artifacts/device-verification/2026-07-03-iphone-us001-016-resumed/iphone-remaining-app-current.png/xml, iphone-us023-us024-us033-profile-scrolled.png/xml。SimulatorのCoreSimulator warningとは別に物理iPhone UI取得は復旧済み。</t>
@@ -4362,11 +4697,7 @@
           <t>PASS: 2026-06-29 web/admin npm run typecheck と npm run build 成功。Next.js buildで管理API route生成まで確認。</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
         <is>
           <t>修正なし: typecheck/buildエラー未検出。</t>
@@ -4377,21 +4708,9 @@
           <t>PASS local retest。本番env/API実動作は未検証。</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T41" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr">
         <is>
           <t>2026-06-29 00:39:51 +0900</t>
@@ -4484,16 +4803,8 @@
           <t>PASS linked DB: db query --linkedで主要table/RPC存在確認成功。PASS functions: contact-support/contact-support-resend-webhook/verify-store-purchase deploy成功。PASS advisors improvement: anon executable SECURITY DEFINERはpreview系3件のみ。Remaining advisors WARN: function search_path、signed-in SECURITY DEFINER、RLS initplan、multiple policies、leaked password protection。 2026-07-03追加: deno check supabase/functions/verify-store-purchase/index.ts、contact-support/index.ts、contact-support-resend-webhook/index.ts は全てPASS。</t>
         </is>
       </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S42" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr">
         <is>
           <t>linked project xocumgxbylmpoobfqows。db pushはremote migration history driftにより不可だったため、必要migrationをdb query --linkedで個別適用。 2026-07-03確認: Supabase vanity domain linbam.supabase.co は未解決で、vanity-subdomains APIはPro/Team/Enterprise plan requiredを返す。現行project ref xocumgxbylmpoobfqowsは到達するが匿名healthは401。</t>
@@ -4912,16 +5223,8 @@
           <t>PASS linked DB: store_purchase_verifications columns/RLS policy確認。PASS Function: verify-store-purchase no-session request is rejected with 401. Remaining: Google Play/App Store sandbox実取引と通知イベント。</t>
         </is>
       </c>
-      <c r="R46" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S46" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
       <c r="T46" t="inlineStr">
         <is>
           <t>実装コミット 7a2aba31。AS系に課金監査ストーリーを追加。</t>
@@ -5340,16 +5643,8 @@
           <t>PASS live send: contact-support POST returned 202 accepted requestId=56d99d04-bbea-4b48-be13-eef62cb1f8d4。PASS DB: delivery_status=sent, delivery_provider=resend, has_message_id=true, delivery_event_type=email.sent。PASS webhook smoke: unsigned webhook returns 401 Invalid webhook secret。15秒後の確認ではdelivered webhook未反映。</t>
         </is>
       </c>
-      <c r="R50" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S50" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
       <c r="T50" t="inlineStr">
         <is>
           <t>Resend配送完了truthはResend側webhook実イベントまたはResend API照会が必要。</t>
@@ -5447,16 +5742,8 @@
           <t>PASS: npx --yes vercel@latest --prod --yes 成功。deployment dpl_8WZa3BBdqQs4f8s8mKcvxzaspVdv / alias https://miyamibu.xyz。PASS: scripts/verify_public_web_release.sh は privacy/account-deletion HTTP 200、assetlinks/AASA ID、Standard / Pro、Google Play Billing、StoreKit、stale no-real-billing文言なしを全て確認。</t>
         </is>
       </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S51" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R51" t="inlineStr"/>
+      <c r="S51" t="inlineStr"/>
       <c r="T51" t="inlineStr">
         <is>
           <t>2026-06-29 live privacy staleはproduction deployで解消。残りはPlay Console final SHA-256など外部Console確認のみ。</t>
@@ -6089,16 +6376,8 @@
           <t>未実施: live Resend APIと管理者セッションが必要。</t>
         </is>
       </c>
-      <c r="R57" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S57" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="R57" t="inlineStr"/>
+      <c r="S57" t="inlineStr"/>
       <c r="T57" t="inlineStr">
         <is>
           <t>AS-006はwebhook反映、AS-009はResend APIへの手動照会。</t>
@@ -6270,66 +6549,79 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>PARTIAL: Render入口からYouTube Shorts/通常動画のRailway委譲asset取得PASS。Instagram Reel/写真/複数投稿もRender本番resolverでasset取得確認済み。iPhone実機でYouTube Shortsの保存、メディアを保存、メディアを開くPASS。Android実機とiPhone全リンク全形式の網羅は未完了。Xは対象外。</t>
+          <t>PASS: Render/Railway本番resolverとAndroid/iPhone実機で、指定TikTok/Instagram/YouTubeリンクの保存、メディア保存、メディアを開く、ビューア表示を確認。Xはユーザー指定どおりメディア保存対象外。</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>physical_android;physical_iphone</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>PASS: Render /health は本番commit cdfbb72418dad30b55bcf4b1dade063b189394c7、youtube.delegateConfigured=true、delegateHost=rinbam-youtube-resolver-production.up.railway.app。Railway /health はYouTube cookie contentConfigured=true。</t>
+          <t>PASS: Render /health は本番commit e083730771fbf268816da78018cb7e52f5018680でYouTube delegate設定済み。Railway /health はYouTube cookie contentConfigured=true。2026-07-07追加: Railwayに a9ce0238 をdeployし、YouTube通常動画は server-download fallback で /files mp4 を返すことを確認。</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>解消済み: Render単体YouTube取得失敗はRailway専用resolverへの委譲で回避。未完了: Androidはadb devices 0件のため最新backend状態の実機メディア保存未確認。iPhoneはYouTube Shortsのみ実機PASSで、Instagram/YouTube通常/複数画像など全リンク網羅は未完了。</t>
+          <t>解消済み: Android実機未接続はPixel 9a 55211JEBF16639接続で解消。iPhone全リンク未網羅はAppium/WDAで再検証し解消。YouTube通常動画のRailway direct proxy 502は、server-download有効時にcached /filesを返す修正で解消。</t>
         </is>
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>FIXED_BACKEND_PARTIAL_DEVICE: scripts/media_resolver_backend.py に MEDIA_RESOLVER_YOUTUBE_DELEGATE_URL 委譲とループ防止を追加。Railway resolverを新規作成し、Render DashboardでMEDIA_RESOLVER_YOUTUBE_DELEGATE_URLを設定。Xはメディア保存対象外として除外。</t>
+          <t>FIXED_BACKEND_AND_DEVICE: AndroidはDetailViewModelでメディア保存押下時に常に再resolveし、VideoResolverでURL中の\%を正規化。BackendはYouTube direct proxyで安全なyt-dlp headersを保持し、server-download有効時はproxyではなくcached /filesを返す。Xは対象外維持。</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>PASS backend: Railway /resolve は YouTube Shorts/通常動画で VIDEO asset + downloadUrl を返す。PASS Render入口: https://rinbam-media-resolver.onrender.com/resolve でも同2件が HTTP 200 ok=true provider=youtube assets=1。PASS iPhone partial: YouTube Shortsを手動追加保存し、詳細でメディアを保存、保存後メディアを開く表示、ビューア表示まで確認。</t>
+          <t>PASS backend: Railway /resolve とRender入口 /resolve でYouTube通常動画が /files/df856baf91a5288eded2bdf5.mp4 を返し、GETで video/mp4 139792928 bytes を取得可能。PASS backend: TikTok、Instagram Reel、Instagram写真、Instagram複数/混在、YouTube Shorts、YouTube通常動画のasset取得確認。PASS local: python3 -m unittest tests/test_media_resolver_backend.py、./gradlew assembleDebug、./gradlew testDebugUnitTest --tests jp.mimac.urlsaver.MediaResolveErrorReasonTest、verify_mobile_ui_contract、verify_canonical_story_tracker、git diff --check。</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>NOT VERIFIED on current physical Android after Render YouTube delegate: adb devices が空のため、jp.miyamibu.urlalbum でYouTube/Instagramメディア保存とメディアを開く操作は未完了。</t>
+          <t>PASS(Android physical Pixel 9a 55211JEBF16639, package jp.miyamibu.urlalbum): 指定6リンクを実機で保存/詳細/メディア保存/メディアを開く/ビューア表示まで確認。TikTok video、Instagram Reel video、Instagram写真複数画像、Instagram混在/動画、YouTube Shorts video、YouTube通常動画 video を確認。Android写真リンクは stale/null asset により一度失敗し、再resolve + URL正規化修正後にPASS。証跡: artifacts/device-verification/2026-07-07-media-e2e/android-*。</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>PARTIAL PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 3d33f82b-f41e-416f-89d3-cbe1f16d93af, bundle com.mibu.codebridge.ios): YouTube Shorts https://youtube.com/shorts/ct-lmvk6mO0 を手動追加で保存し、ホームカード表示、詳細のメディアを保存表示、押下後メディアを開くへの切替、メディアビューア表示を確認。証跡: artifacts/device-verification/2026-07-05-final-gates/iphone-after-youtube-save-3.png/xml, iphone-youtube-detail.png/xml, iphone-after-media-save.png/xml, iphone-media-viewer.png/xml。未完了: iPhoneのInstagram Reel/写真/複数投稿、YouTube通常動画、TikTokの全リンク網羅。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA sessions d291e3f9-0568-4081-828b-ef0bb130f8c3 and 893decce-78d6-4d47-9096-3b04d9875ac1, bundle com.mibu.codebridge.ios): 検証用共有元アプリから指定6リンクを共有し、各URLが共有シート/りんばむ共有拡張に出ていることと保存しましたを確認。TikTok、Instagram Reel、Instagram写真複数画像、Instagram混在、YouTube Shorts、YouTube通常動画を本体詳細でメディア保存し、保存後メディアを開くへ切替、ビューア表示まで確認。YouTube通常動画はRailway /files修正後に最終PASS。証跡: artifacts/device-verification/2026-07-07-media-e2e/iphone-*retry3*, iphone-*retry4*, iphone-youtube-normal-*railway-files*。</t>
         </is>
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>2026-07-05 23:59更新。Railway project rinbam-youtube-resolver / domain https://rinbam-youtube-resolver-production.up.railway.app をYouTube専用delegateとして作成。Render入口は維持。Render/Railway検証JSONは artifacts/render-verification/2026-07-05-final-gates/ に保存。Android未接続とiPhone全リンク未網羅は完了扱いにしない。</t>
+          <t>2026-07-07更新: Railway project rinbam-youtube-resolver へ a9ce0238 をdeploy。Render入口は維持。検証JSON: artifacts/render-verification/2026-07-07-media-e2e/。実機証跡: artifacts/device-verification/2026-07-07-media-e2e/。未追跡artifactは証跡としてローカル保持し、ソースコミットには含めない。</t>
         </is>
       </c>
       <c r="U59" t="inlineStr">
         <is>
-          <t>2026-07-05 23:59:00 +0900</t>
+          <t>2026-07-08 00:25:00 +0900</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:U59"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6387,7 +6679,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -6399,7 +6691,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
     </row>
@@ -6440,14 +6732,10 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>US-042</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6457,14 +6745,10 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>US-042</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6477,11 +6761,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6569,5 +6849,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement Chapter 13 ChatGPT handoff and release hardening
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U59"/>
+  <dimension ref="A1:U60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3830,7 +3830,11 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P32" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -3841,8 +3845,16 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T32" t="inlineStr">
         <is>
           <t>秘密値は扱わない</t>
@@ -3925,7 +3937,11 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P33" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -3936,9 +3952,21 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U33" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -4016,7 +4044,11 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P34" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -4027,8 +4059,16 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T34" t="inlineStr">
         <is>
           <t>実送信は承認なしにしない</t>
@@ -4111,7 +4151,11 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P35" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -4122,9 +4166,21 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
-      <c r="T35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U35" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -4202,7 +4258,11 @@
           <t>PASS: web/admin npm run typecheck と npm run build 成功。 / BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P36" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -4213,9 +4273,21 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U36" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -4293,7 +4365,11 @@
           <t>BLOCKED_LOCAL: supabase db lint --local は 127.0.0.1:55422 接続拒否。ローカルDB未起動。本番/linked DBは秘密値なしで未接続。 / PASS: web/admin npm run typecheck と npm run build 成功。</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P37" t="inlineStr">
         <is>
           <t>修正なし: エラー未検出。</t>
@@ -4304,9 +4380,21 @@
           <t>再テスト不要: 変更なし。</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
-      <c r="T37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U37" t="inlineStr">
         <is>
           <t>2026-06-27 15:51:33 +0900</t>
@@ -4511,7 +4599,11 @@
           <t>PASS(Android physical Pixel 9a 55211JEBF16639): jp.miyamibu.urlalbum 起動、ホーム、下部5アクション、使い方リスト、戻る復帰をXML/PNGで確認。</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr"/>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T39" t="inlineStr">
         <is>
           <t>connectedDebugAndroidTestは通常端末では承認なし実行しない。テスト専用AVDでは2026-06-29に実行済み。2026-06-29にステータスをPASSからLOCAL_PASS_WITH_CONNECTED_TEST_GAPへ修正し、未検証ゲートを分離。 2026-06-29 connectedDebugAndroidTestをテスト専用AVDで実行し成功。</t>
@@ -4609,7 +4701,11 @@
           <t>PASS local retest: MetadataStatusTextTests成功、duplicate display_nameログなし、container_create_or_lookupログなし。 2026-07-03追加: xcodebuild selected local/simulator tests PASS 26 tests。 2026-07-03 07:12追加 iPhone physical via Appium/WDA: PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA + devicectl): com.mibu.codebridge.ios 1.0.11(11) を実機に上書きインストール済み。Appium/WDAでホーム、共有タグサインイン案内、プロフィール/プラン画面のUIツリーとスクリーンショット取得に成功。証跡: artifacts/device-verification/2026-07-03-iphone-us001-016-resumed/iphone-remaining-app-current.png/xml, iphone-us023-us024-us033-profile-scrolled.png/xml。SimulatorのCoreSimulator warningとは別に物理iPhone UI取得は復旧済み。</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="S40" t="inlineStr">
         <is>
           <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA + devicectl): com.mibu.codebridge.ios 1.0.11(11) を実機に上書きインストール済み。Appium/WDAでホーム、共有タグサインイン案内、プロフィール/プラン画面のUIツリーとスクリーンショット取得に成功。証跡: artifacts/device-verification/2026-07-03-iphone-us001-016-resumed/iphone-remaining-app-current.png/xml, iphone-us023-us024-us033-profile-scrolled.png/xml。SimulatorのCoreSimulator warningとは別に物理iPhone UI取得は復旧済み。</t>
@@ -4697,7 +4793,11 @@
           <t>PASS: 2026-06-29 web/admin npm run typecheck と npm run build 成功。Next.js buildで管理API route生成まで確認。</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="P41" t="inlineStr">
         <is>
           <t>修正なし: typecheck/buildエラー未検出。</t>
@@ -4708,9 +4808,21 @@
           <t>PASS local retest。本番env/API実動作は未検証。</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
-      <c r="T41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="U41" t="inlineStr">
         <is>
           <t>2026-06-29 00:39:51 +0900</t>
@@ -4803,8 +4915,16 @@
           <t>PASS linked DB: db query --linkedで主要table/RPC存在確認成功。PASS functions: contact-support/contact-support-resend-webhook/verify-store-purchase deploy成功。PASS advisors improvement: anon executable SECURITY DEFINERはpreview系3件のみ。Remaining advisors WARN: function search_path、signed-in SECURITY DEFINER、RLS initplan、multiple policies、leaked password protection。 2026-07-03追加: deno check supabase/functions/verify-store-purchase/index.ts、contact-support/index.ts、contact-support-resend-webhook/index.ts は全てPASS。</t>
         </is>
       </c>
-      <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T42" t="inlineStr">
         <is>
           <t>linked project xocumgxbylmpoobfqows。db pushはremote migration history driftにより不可だったため、必要migrationをdb query --linkedで個別適用。 2026-07-03確認: Supabase vanity domain linbam.supabase.co は未解決で、vanity-subdomains APIはPro/Team/Enterprise plan requiredを返す。現行project ref xocumgxbylmpoobfqowsは到達するが匿名healthは401。</t>
@@ -5223,8 +5343,16 @@
           <t>PASS linked DB: store_purchase_verifications columns/RLS policy確認。PASS Function: verify-store-purchase no-session request is rejected with 401. Remaining: Google Play/App Store sandbox実取引と通知イベント。</t>
         </is>
       </c>
-      <c r="R46" t="inlineStr"/>
-      <c r="S46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T46" t="inlineStr">
         <is>
           <t>実装コミット 7a2aba31。AS系に課金監査ストーリーを追加。</t>
@@ -5643,8 +5771,16 @@
           <t>PASS live send: contact-support POST returned 202 accepted requestId=56d99d04-bbea-4b48-be13-eef62cb1f8d4。PASS DB: delivery_status=sent, delivery_provider=resend, has_message_id=true, delivery_event_type=email.sent。PASS webhook smoke: unsigned webhook returns 401 Invalid webhook secret。15秒後の確認ではdelivered webhook未反映。</t>
         </is>
       </c>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T50" t="inlineStr">
         <is>
           <t>Resend配送完了truthはResend側webhook実イベントまたはResend API照会が必要。</t>
@@ -5742,8 +5878,16 @@
           <t>PASS: npx --yes vercel@latest --prod --yes 成功。deployment dpl_8WZa3BBdqQs4f8s8mKcvxzaspVdv / alias https://miyamibu.xyz。PASS: scripts/verify_public_web_release.sh は privacy/account-deletion HTTP 200、assetlinks/AASA ID、Standard / Pro、Google Play Billing、StoreKit、stale no-real-billing文言なしを全て確認。</t>
         </is>
       </c>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T51" t="inlineStr">
         <is>
           <t>2026-06-29 live privacy staleはproduction deployで解消。残りはPlay Console final SHA-256など外部Console確認のみ。</t>
@@ -6376,8 +6520,16 @@
           <t>未実施: live Resend APIと管理者セッションが必要。</t>
         </is>
       </c>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="T57" t="inlineStr">
         <is>
           <t>AS-006はwebhook反映、AS-009はResend APIへの手動照会。</t>
@@ -6600,6 +6752,113 @@
       <c r="U59" t="inlineStr">
         <is>
           <t>2026-07-08 00:25:00 +0900</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>CH-013</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>ユーザー</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Android/iOS</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>AI引き渡し</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>第13章 ChatGPT活用例の受け側契約</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>ExportRepository.kt; ExportArchiveBuilder.swift; ExportScreen.kt; ExportSheet.swift; docs/ai/chapter13-chatgpt-use-cases.md</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Google Doc第13章の34項目を添付後のChatGPTで依頼できる例として確認し、りんばむ側は自作タグ選択・対象/出力内容確認・ZIP作成・OS共有までに限定する。</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>README_FOR_AI.mdに34項目を1から34まで含める。質問入力・自動入力・自動送信・OpenAI API/OAuth/MCPは含めない。共有前に未知の秘密が残る可能性を警告し明示確認を要求する.</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Android/iOS単体テスト; README 34項目照合; iPhone Appium/WDA composer添付確認; Androidは実機/AVD接続後に同一手順を再実行。</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>提出binaryのAndroid/iOS両方で同じ34項目と責務境界が表示されること。</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>IMPLEMENTED_LOCAL_WITH_DEVICE_GATES</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>android_device;distribution_signing;public_privacy;store_console</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Android/iOS source and unit tests pass. iPhone physical reaches normal ChatGPT composer with ZIP attached and question field empty; Android physical unavailable.</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>未署名AAB・Android物理E2E・iOS Distribution/TestFlight・公開Privacy反映・Store申告は外部ゲート。</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>FAIL_CLOSED_AND_BOUNDARY_HARDENED</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>iOS saved-session plus unavailable config now fails closed. Android Release Ads references removed and ChatGPT share intent/cache/25MiB/10000-entry guards added. Redaction now occurs before excerpt clipping with boundary regression tests。未実施: Android物理端末/AVDで直接共有とchooser fallback、Release cold start。iOS最終送信は仕様上実施しない。</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>NOT VERIFIED on Android physical: device/AVD unavailable.</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>PASS iPhone physical via Appium/WDA: ZIP attachment in normal ChatGPT composer and empty question field; send intentionally not tapped.</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Chapter 13 is a receiving-side use-case list・not 34 in-app AI features. Canonical fixture: docs/ai/chapter13-chatgpt-use-cases.md.</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>2026-07-18 00:00:00 +0900</t>
         </is>
       </c>
     </row>
@@ -6679,7 +6938,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -6735,7 +6994,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6748,7 +7011,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6761,7 +7028,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6788,12 +7059,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>US-002,US-006,US-014,US-015,US-016,US-017,US-021,US-023,US-029,US-032,US-033,AS-007,ES-006,US-040,TS-001</t>
+          <t>US-002,US-006,US-014,US-015,US-016,US-017,US-021,US-023,US-029,US-032,US-033,AS-007,ES-006,US-040,TS-001,CH-013</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(qa): record live delivery and iPhone evidence
</commit_message>
<xml_diff>
--- a/docs/qa/rinbam_canonical_story_status.xlsx
+++ b/docs/qa/rinbam_canonical_story_status.xlsx
@@ -3170,7 +3170,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>PARTIAL: local export testsと両実機の設定画面PASS、物理共有/ファイル保存E2Eは未検証</t>
+          <t>PARTIAL: local export testsと両実機の設定画面PASS。iPhoneは実書き出しからiOS共有シート表示・未送信で閉じるまでPASS。Android出力実行E2Eは未検証。</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -3180,7 +3180,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>android_device;iphone_device</t>
+          <t>android_device</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3190,17 +3190,17 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>物理Android/iPhoneでの共有シート、ファイル保存、ファイル受け渡し先アプリでの実確認は未検証。iOS simulator test中にApp Group entitlement警告と重複display_name migrationログあり、テスト失敗はなし。</t>
+          <t>物理Androidでの書き出し実行、共有シート、ファイル保存、受け渡し先アプリ確認は未検証。iPhoneはUIActivityViewController表示まで実行済み。</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>修正なし: ローカルテスト上のエラー未検出。台帳code_basisに共有シート/保存先実装を補強。</t>
+          <t>DEVICE_EVIDENCE_UPDATED: iPhone物理実機でZIP書き出しとUIActivityViewController表示を確認。外部送信は行わず閉じてホーム復帰。</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>PASS local retest: Android export targeted tests、iOS export/filter targeted tests成功。物理共有先は未実施。</t>
+          <t>PASS local retest: Android export targeted tests、iOS export/filter targeted tests成功。物理共有先は未実施。 PASS iPhone physical 2026-08-23/24: ZIP・共有シートを選び「書き出す」を実行、iOS UIActivityViewControllerでAirDrop/コピーを確認し、送信せず閉じてホームへ復帰。</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -3210,17 +3210,17 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>PASS/PARTIAL(iPhone physical 00008101-00066D96340A001E via Appium/WDA session 8c957f69-e6f0-412a-9d20-816728e11a1b): エクスポート画面で「ZIP」「JSON」「共有シート」「ファイルに保存」「書き出す」を確認。UIActivityViewController/fileExporter実行は未実施。証跡: iphone-ui-loop-export-open-final.png/xml。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E, bundle com.mibu.codebridge.ios 1.0.18(20), Appium/WDA session b7d4dca2-079d-4186-bd43-866f79ecec8f): エクスポート画面でZIP・共有シートを選び「書き出す」を実行。iOS共有シートにAirDrop/コピーが表示され、外部送信せず閉じ、エクスポート画面とホームへ正常復帰。証跡: artifacts/device-verification/2026-08-23-final/iphone-appium/11-export-sheet.png/xml相当、12-system-share-sheet.png/xml、13-home-final.png/xml。</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>実ファイル生成、共有先アプリ、ファイル保存先確認は次ループで実施。</t>
+          <t>iPhoneの実ファイル生成と共有シート起動は物理PASS。外部送信は仕様・データ保護のため実施せず。Android物理出力E2Eのみ継続。</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>2026-08-11 11:02:17 +0900</t>
+          <t>2026-08-24 19:59:34 +0900</t>
         </is>
       </c>
     </row>
@@ -5738,17 +5738,17 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>PASS_RESEND_SENT_WITH_DELIVERY_EVENT_GAP</t>
+          <t>PASS_LIVE_RESEND_DELIVERED_AND_AUDITED: 本番contact-support canaryが202 accepted、同一idempotency key再送で同一requestId、Resend email.delivered、outbox sent、message id保存、payload scrub、監査更新まで確認。</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>BLOCKED_EXTERNAL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>supabase_auth;resend_live</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -5758,17 +5758,17 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>Resend delivered/bounced/complained等の実webhookイベント反映は未確認。問い合わせ送信、Resend accepted相当のemail.sent、DB監査row、message id保存は確認済み。</t>
+          <t>確認した範囲ではなし。Resend署名済みemail.deliveredイベントが本番DBへ反映され、provider配送完了と監査更新を確認。</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>FIXED_LIVE: contact-support-resend-webhookを本番deploy。contact-support Functionをpublic.contact_support_requests契約へ修正し、問い合わせ本文/メール/名前の原文を監査DBへ保存しない形へ変更。Resend message idを保存し、webhookが後続更新できる状態にした。</t>
+          <t>FIXED_LIVE_AND_DELIVERY_VERIFIED</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>PASS live send: contact-support POST returned 202 accepted requestId=56d99d04-bbea-4b48-be13-eef62cb1f8d4。PASS DB: delivery_status=sent, delivery_provider=resend, has_message_id=true, delivery_event_type=email.sent。PASS webhook smoke: unsigned webhook returns 401 Invalid webhook secret。15秒後の確認ではdelivered webhook未反映。</t>
+          <t>PASS live 2026-08-23/24: contact-support POSTは202 accepted、requestId=d5c3903e-c565-4021-9e0c-425f0f776ccc。同一Idempotency-Key再送も同一requestIdで二重送信なし。PASS linked DB: delivery_status=delivered、delivery_event_type=email.delivered、delivery_message_idあり、outbox state=sent、attempts=1、payload={}、payload_scrubbed_atあり。</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -5783,12 +5783,12 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>Resend配送完了truthはResend側webhook実イベントまたはResend API照会が必要。</t>
+          <t>本番Resend delivery truthを署名済みemail.delivered webhookの実DB反映で確認。問い合わせ本文・氏名・メールは合成canaryのみを使用し、outbox送信後scrub済み。</t>
         </is>
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-29 07:25:00 +0900</t>
+          <t>2026-08-24 19:57:29 +0900</t>
         </is>
       </c>
     </row>
@@ -5952,17 +5952,17 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>PARTIAL: Android実データ検索と両OSunit/UI操作PASS、iPhone実データ絞り込みE2Eは未検証</t>
+          <t>PASS: Android/iPhone実データ検索、両OS unit、検索表示・入力・絞り込み・終了後ホーム復帰を確認。</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>iphone_device</t>
+          <t>none</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -5972,17 +5972,17 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>iPhone物理実機での実データ絞り込み、no-result、検索から詳細/戻るの連続操作は未検証。Appium/usbmuxd未復旧のため追加操作証跡なし。</t>
+          <t>確認した範囲ではなし。no-resultと検索結果から詳細遷移の追加回帰は将来拡張であり、正準受入の実データ絞り込みは両物理端末で確認済み。</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>FIXED_LOCAL: Android/iOSの検索対象を正準仕様へ拡張。AndroidはfetchedAuthorName/fetchedBody/bodySummary/description/memo/service labelを追加し、タグ割当参照をLOCAL_ONLY限定から可視タグ名照合用の全割当へ拡張。iOSは既存の本文/メモ/投稿主名検索にservice labelを追加。</t>
+          <t>FIXED_LOCAL_AND_BOTH_PHYSICAL_DEVICES_VERIFIED</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>PASS local: Android MainListViewModelTestで本文/投稿内容、メモ、投稿主名、サービス名、割当共有タグ名検索を追加確認。PASS local: iOS ServiceFilterTestsで本文/投稿内容、メモ、投稿主名、サービス名検索を追加確認。PASS Android physical: IANA実データ検索で1件絞り込み確認。</t>
+          <t>PASS local: Android MainListViewModelTestで本文/投稿内容、メモ、投稿主名、サービス名、割当共有タグ名検索を追加確認。PASS local: iOS ServiceFilterTestsで本文/投稿内容、メモ、投稿主名、サービス名検索を追加確認。PASS Android physical: IANA実データ検索で1件絞り込み確認。 PASS iPhone physical 2026-08-23/24: 検索欄へexampleを入力し、example.comの実データ1件へ絞り込み。検索終了後に通常ホームと5アクションへ復帰。</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -5992,17 +5992,17 @@
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>PASS(iPhone physical 00008101-00066D96340A001E via Appium/WDA session cca5fad7-b2ae-491d-a4ac-95499e1ed33b): 検索ボタンからTextField表示、rinbamtest入力、クリアボタン表示、クリア後ホーム復帰を確認。証跡: artifacts/device-verification/2026-06-29/iphone-us037-search-open.png/source.xml, iphone-us037-search-input.png/source.xml, iphone-us037-search-cleared.png/source.xml。</t>
+          <t>PASS(iPhone physical 00008101-00066D96340A001E, bundle com.mibu.codebridge.ios 1.0.18(20), Appium/WDA session b7d4dca2-079d-4186-bd43-866f79ecec8f): 検索欄へexampleを入力し、example.comカードだけが表示される実データ絞り込みを確認。検索終了後に通常ホームと5アクションへ復帰。証跡: artifacts/device-verification/2026-08-23-final/iphone-appium/10-search-example.png/xml、13-home-final.png/xml。</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
         <is>
-          <t>Androidでは既存IANAカードを使った実データ検索まで物理PASS。iPhone側の実データ絞り込みはAppium/usbmuxd未復旧のため未検証。共有タグ名検索の物理実データはSupabase/live共有タグ状態が必要。動画/メディア保存設定は今回後回し。</t>
+          <t>AndroidのIANA検索とiPhoneのexample検索で、両物理端末の実データ絞り込みを確認済み。共有タグ名検索のlive状態は共有タグ個別ストーリーで追跡する。</t>
         </is>
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2026-08-11 11:02:17 +0900</t>
+          <t>2026-08-24 19:59:34 +0900</t>
         </is>
       </c>
     </row>
@@ -6902,7 +6902,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>23</t>
         </is>
       </c>
     </row>
@@ -6926,7 +6926,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -6938,7 +6938,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>27</t>
         </is>
       </c>
     </row>
@@ -6996,12 +6996,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>US-013,US-021,US-025,US-037</t>
+          <t>US-013,US-021</t>
         </is>
       </c>
     </row>
@@ -7030,12 +7030,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>US-016,US-017,US-018,US-019,US-020,US-022,US-023,US-024,AS-001,AS-002,AS-003,AS-004,AS-005,AS-006,ES-005,US-032,US-033,AS-007,AS-008,US-039,AS-009</t>
+          <t>US-016,US-017,US-018,US-019,US-020,US-022,US-023,US-024,AS-001,AS-002,AS-003,AS-004,AS-005,AS-006,ES-005,US-032,US-033,AS-007,US-039,AS-009</t>
         </is>
       </c>
     </row>
@@ -7064,12 +7064,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AS-003,AS-006,AS-008,AS-009</t>
+          <t>AS-003,AS-006,AS-009</t>
         </is>
       </c>
     </row>

</xml_diff>